<commit_message>
Updated codebase Workday playwright..
</commit_message>
<xml_diff>
--- a/Data/Hires/Copy of Workday_NewHire_Slovenia_Regression_PK17 End To End May 23_.xlsx
+++ b/Data/Hires/Copy of Workday_NewHire_Slovenia_Regression_PK17 End To End May 23_.xlsx
@@ -1,20 +1,37 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
-  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="27928"/>
+  <workbookPr filterPrivacy="1"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0633199B-1006-47FF-8507-4D8842A87477}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet sheetId="1" name="Sheet2" state="visible" r:id="rId4"/>
+    <sheet name="Sheet2" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="171027"/>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase">Sheet2!$A$1:$BV$21</definedName>
+  </definedNames>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1165" uniqueCount="197">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1191" uniqueCount="223">
   <si>
     <t>TestCaseIDs</t>
   </si>
@@ -481,7 +498,13 @@
     <t>Test11</t>
   </si>
   <si>
-    <t>TestTwentyFive</t>
+    <t>10699353</t>
+  </si>
+  <si>
+    <t>Maddison</t>
+  </si>
+  <si>
+    <t>Dooley</t>
   </si>
   <si>
     <t>070-417-635</t>
@@ -496,424 +519,252 @@
     <t>Test12</t>
   </si>
   <si>
-    <t xml:space="preserve">Test failed for 'Omer Shields' Employee:{10699346}TimeoutError: locator.click: Timeout 30000ms exceeded.
-Call log:
-  [2m- waiting for locator('//div[@data-automation-id="tooltipsWrapper"]/button[@data-automation-id="inbox_preview"]').first()[22m
-[2m  -   locator resolved to &lt;button class="wdappchrome-w" data-automation-id="inbox_…&gt;…&lt;/button&gt;[22m
-[2m  - attempting click action[22m
-[2m  -   waiting for element to be visible, enabled and stable[22m
-[2m  -   element is not visible[22m
-[2m  - retrying click action, attempt #1[22m
-[2m  -   waiting for element to be visible, enabled and stable[22m
-[2m  -   element is not visible[22m
-[2m  - retrying click action, attempt #2[22m
-[2m  -   waiting 20ms[22m
-[2m  -   waiting for element to be visible, enabled and stable[22m
-[2m  -   element is not visible[22m
-[2m  - retrying click action, attempt #3[22m
-[2m  -   waiting 100ms[22m
-[2m  -   waiting for element to be visible, enabled and stable[22m
-[2m  -   element is not visible[22m
-[2m  - retrying click action, attempt #4[22m
-[2m  -   waiting 100ms[22m
-[2m  -   waiting for element to be visible, enabled and stable[22m
-[2m  -   element is not visible[22m
-[2m  - retrying click action, attempt #5[22m
-[2m  -   waiting 500ms[22m
-[2m  -   waiting for element to be visible, enabled and stable[22m
-[2m  -   element is not visible[22m
-[2m  - retrying click action, attempt #6[22m
-[2m  -   waiting 500ms[22m
-[2m  -   waiting for element to be visible, enabled and stable[22m
-[2m  -   element is not visible[22m
-[2m  - retrying click action, attempt #7[22m
-[2m  -   waiting 500ms[22m
-[2m  -   waiting for element to be visible, enabled and stable[22m
-[2m  -   element is not visible[22m
-[2m  - retrying click action, attempt #8[22m
-[2m  -   waiting 500ms[22m
-[2m  -   waiting for element to be visible, enabled and stable[22m
-[2m  -   element is not visible[22m
-[2m  - retrying click action, attempt #9[22m
-[2m  -   waiting 500ms[22m
-[2m  -   waiting for element to be visible, enabled and stable[22m
-[2m  -   element is not visible[22m
-[2m  - retrying click action, attempt #10[22m
-[2m  -   waiting 500ms[22m
-[2m  -   waiting for element to be visible, enabled and stable[22m
-[2m  -   element is not visible[22m
-[2m  - retrying click action, attempt #11[22m
-[2m  -   waiting 500ms[22m
-[2m  -   waiting for element to be visible, enabled and stable[22m
-[2m  -   element is not visible[22m
-[2m  - retrying click action, attempt #12[22m
-[2m  -   waiting 500ms[22m
-[2m  -   waiting for element to be visible, enabled and stable[22m
-[2m  -   element is not visible[22m
-[2m  - retrying click action, attempt #13[22m
-[2m  -   waiting 500ms[22m
-[2m  -   waiting for element to be visible, enabled and stable[22m
-[2m  -   element is not visible[22m
-[2m  - retrying click action, attempt #14[22m
-[2m  -   waiting 500ms[22m
-[2m  -   waiting for element to be visible, enabled and stable[22m
-[2m  -   element is not visible[22m
-[2m  - retrying click action, attempt #15[22m
-[2m  -   waiting 500ms[22m
-[2m  -   waiting for element to be visible, enabled and stable[22m
-[2m  -   element is not visible[22m
-[2m  - retrying click action, attempt #16[22m
-[2m  -   waiting 500ms[22m
-[2m  -   waiting for element to be visible, enabled and stable[22m
-[2m  -   element is not visible[22m
-[2m  - retrying click action, attempt #17[22m
-[2m  -   waiting 500ms[22m
-[2m  -   waiting for element to be visible, enabled and stable[22m
-[2m  -   element is not visible[22m
-[2m  - retrying click action, attempt #18[22m
-[2m  -   waiting 500ms[22m
-[2m  -   waiting for element to be visible, enabled and stable[22m
-[2m  -   element is not visible[22m
-[2m  - retrying click action, attempt #19[22m
-[2m  -   waiting 500ms[22m
-[2m  -   waiting for element to be visible, enabled and stable[22m
-[2m  -   element is not visible[22m
-[2m  - retrying click action, attempt #20[22m
-[2m  -   waiting 500ms[22m
-[2m  -   waiting for element to be visible, enabled and stable[22m
-[2m  -   element is not visible[22m
-[2m  - retrying click action, attempt #21[22m
-[2m  -   waiting 500ms[22m
-[2m  -   waiting for element to be visible, enabled and stable[22m
-[2m  -   element is not visible[22m
-[2m  - retrying click action, attempt #22[22m
-[2m  -   waiting 500ms[22m
-[2m  -   waiting for element to be visible, enabled and stable[22m
-[2m  -   element is not visible[22m
-[2m  - retrying click action, attempt #23[22m
-[2m  -   waiting 500ms[22m
-[2m  -   waiting for element to be visible, enabled and stable[22m
-[2m  -   element is not visible[22m
-[2m  - retrying click action, attempt #24[22m
-[2m  -   waiting 500ms[22m
-[2m  -   waiting for element to be visible, enabled and stable[22m
-[2m  -   element is not visible[22m
-[2m  - retrying click action, attempt #25[22m
-[2m  -   waiting 500ms[22m
-[2m  -   waiting for element to be visible, enabled and stable[22m
-[2m  -   element is not visible[22m
-[2m  - retrying click action, attempt #26[22m
-[2m  -   waiting 500ms[22m
-[2m  -   waiting for element to be visible, enabled and stable[22m
-[2m  -   element is not visible[22m
-[2m  - retrying click action, attempt #27[22m
-[2m  -   waiting 500ms[22m
-[2m  -   waiting for element to be visible, enabled and stable[22m
-[2m  -   element is not visible[22m
-[2m  - retrying click action, attempt #28[22m
-[2m  -   waiting 500ms[22m
-[2m  -   waiting for element to be visible, enabled and stable[22m
-[2m  -   element is not visible[22m
-[2m  - retrying click action, attempt #29[22m
-[2m  -   waiting 500ms[22m
-[2m  -   waiting for element to be visible, enabled and stable[22m
-[2m  -   element is not visible[22m
-[2m  - retrying click action, attempt #30[22m
-[2m  -   waiting 500ms[22m
-[2m  -   waiting for element to be visible, enabled and stable[22m
-[2m  -   element is not visible[22m
-[2m  - retrying click action, attempt #31[22m
-[2m  -   waiting 500ms[22m
-[2m  -   waiting for element to be visible, enabled and stable[22m
-[2m  -   element is not visible[22m
-[2m  - retrying click action, attempt #32[22m
-[2m  -   waiting 500ms[22m
-[2m  -   waiting for element to be visible, enabled and stable[22m
-[2m  -   element is not visible[22m
-[2m  - retrying click action, attempt #33[22m
-[2m  -   waiting 500ms[22m
-[2m  -   waiting for element to be visible, enabled and stable[22m
-[2m  -   element is not visible[22m
-[2m  - retrying click action, attempt #34[22m
-[2m  -   waiting 500ms[22m
-[2m  -   waiting for element to be visible, enabled and stable[22m
-[2m  -   element is not visible[22m
-[2m  - retrying click action, attempt #35[22m
-[2m  -   waiting 500ms[22m
-[2m  -   waiting for element to be visible, enabled and stable[22m
-[2m  -   element is not visible[22m
-[2m  - retrying click action, attempt #36[22m
-[2m  -   waiting 500ms[22m
-[2m  -   waiting for element to be visible, enabled and stable[22m
-[2m  -   element is not visible[22m
-[2m  - retrying click action, attempt #37[22m
-[2m  -   waiting 500ms[22m
-[2m  -   waiting for element to be visible, enabled and stable[22m
-[2m  -   element is not visible[22m
-[2m  - retrying click action, attempt #38[22m
-[2m  -   waiting 500ms[22m
-[2m  -   waiting for element to be visible, enabled and stable[22m
-[2m  -   element is not visible[22m
-[2m  - retrying click action, attempt #39[22m
-[2m  -   waiting 500ms[22m
-[2m  -   waiting for element to be visible, enabled and stable[22m
-[2m  -   element is not visible[22m
-[2m  - retrying click action, attempt #40[22m
-[2m  -   waiting 500ms[22m
-[2m  -   waiting for element to be visible, enabled and stable[22m
-[2m  -   element is not visible[22m
-[2m  - retrying click action, attempt #41[22m
-[2m  -   waiting 500ms[22m
-[2m  -   waiting for element to be visible, enabled and stable[22m
-[2m  -   element is not visible[22m
-[2m  - retrying click action, attempt #42[22m
-[2m  -   waiting 500ms[22m
-[2m  -   waiting for element to be visible, enabled and stable[22m
-[2m  -   element is not visible[22m
-[2m  - retrying click action, attempt #43[22m
-[2m  -   waiting 500ms[22m
-[2m  -   waiting for element to be visible, enabled and stable[22m
-[2m  -   element is not visible[22m
-[2m  - retrying click action, attempt #44[22m
-[2m  -   waiting 500ms[22m
-[2m  -   waiting for element to be visible, enabled and stable[22m
-[2m  -   element is not visible[22m
-[2m  - retrying click action, attempt #45[22m
-[2m  -   waiting 500ms[22m
-[2m  -   waiting for element to be visible, enabled and stable[22m
-[2m  -   element is not visible[22m
-[2m  - retrying click action, attempt #46[22m
-[2m  -   waiting 500ms[22m
-[2m  -   waiting for element to be visible, enabled and stable[22m
-[2m  -   element is not visible[22m
-[2m  - retrying click action, attempt #47[22m
-[2m  -   waiting 500ms[22m
-[2m  -   waiting for element to be visible, enabled and stable[22m
-[2m  -   element is not visible[22m
-[2m  - retrying click action, attempt #48[22m
-[2m  -   waiting 500ms[22m
-[2m  -   waiting for element to be visible, enabled and stable[22m
-[2m  -   element is not visible[22m
-[2m  - retrying click action, attempt #49[22m
-[2m  -   waiting 500ms[22m
-[2m  -   waiting for element to be visible, enabled and stable[22m
-[2m  -   element is not visible[22m
-[2m  - retrying click action, attempt #50[22m
-[2m  -   waiting 500ms[22m
-[2m  -   waiting for element to be visible, enabled and stable[22m
-[2m  -   element is not visible[22m
-[2m  - retrying click action, attempt #51[22m
-[2m  -   waiting 500ms[22m
-[2m  -   waiting for element to be visible, enabled and stable[22m
-[2m  -   element is not visible[22m
-[2m  - retrying click action, attempt #52[22m
-[2m  -   waiting 500ms[22m
-[2m  -   waiting for element to be visible, enabled and stable[22m
-[2m  -   element is not visible[22m
-[2m  - retrying click action, attempt #53[22m
-[2m  -   waiting 500ms[22m
-[2m  -   waiting for element to be visible, enabled and stable[22m
-[2m  -   element is not visible[22m
-[2m  - retrying click action, attempt #54[22m
-[2m  -   waiting 500ms[22m
-[2m  -   waiting for element to be visible, enabled and stable[22m
-[2m  -   element is not visible[22m
-[2m  - retrying click action, attempt #55[22m
-[2m  -   waiting 500ms[22m
-[2m  -   waiting for element to be visible, enabled and stable[22m
-[2m  -   element is not visible[22m
-[2m  - retrying click action, attempt #56[22m
-[2m  -   waiting 500ms[22m
-[2m  -   waiting for element to be visible, enabled and stable[22m
-[2m  -   element is not visible[22m
-[2m  - retrying click action, attempt #57[22m
-[2m  -   waiting 500ms[22m
-[2m  -   waiting for element to be visible, enabled and stable[22m
-[2m  -   element is not visible[22m
-[2m  - retrying click action, attempt #58[22m
-[2m  -   waiting 500ms[22m
-[2m  -   waiting for element to be visible, enabled and stable[22m
-[2m  -   element is not visible[22m
-[2m  - retrying click action, attempt #59[22m
-[2m  -   waiting 500ms[22m
-[2m  -   waiting for element to be visible, enabled and stable[22m
-[2m  -   element is not visible[22m
-[2m  - retrying click action, attempt #60[22m
-[2m  -   waiting 500ms[22m
-</t>
+    <t>10699356</t>
+  </si>
+  <si>
+    <t>Ivy</t>
+  </si>
+  <si>
+    <t>Fadel</t>
+  </si>
+  <si>
+    <t>070-417-636</t>
+  </si>
+  <si>
+    <t>07 Footwear</t>
+  </si>
+  <si>
+    <t>Test13</t>
+  </si>
+  <si>
+    <t>10699358</t>
+  </si>
+  <si>
+    <t>Gianni</t>
+  </si>
+  <si>
+    <t>Bechtelar</t>
+  </si>
+  <si>
+    <t>070-417-637</t>
+  </si>
+  <si>
+    <t>08 Ladieswear</t>
+  </si>
+  <si>
+    <t>Test14</t>
+  </si>
+  <si>
+    <t>10699371</t>
+  </si>
+  <si>
+    <t>Alejandra</t>
+  </si>
+  <si>
+    <t>Keeling</t>
+  </si>
+  <si>
+    <t>070-417-638</t>
+  </si>
+  <si>
+    <t>6 Days (Slovenia)</t>
+  </si>
+  <si>
+    <t>11 Household</t>
+  </si>
+  <si>
+    <t>Test15</t>
+  </si>
+  <si>
+    <t>10699361</t>
+  </si>
+  <si>
+    <t>Jerome</t>
+  </si>
+  <si>
+    <t>Johnson</t>
+  </si>
+  <si>
+    <t>070-417-639</t>
+  </si>
+  <si>
+    <t>15 Children's Accessories</t>
+  </si>
+  <si>
+    <t>Test16</t>
+  </si>
+  <si>
+    <t>10699363</t>
+  </si>
+  <si>
+    <t>Jaeden</t>
+  </si>
+  <si>
+    <t>Hermiston</t>
+  </si>
+  <si>
+    <t>070-417-640</t>
+  </si>
+  <si>
+    <t>23 Health &amp; Beauty</t>
+  </si>
+  <si>
+    <t>Test17</t>
+  </si>
+  <si>
+    <t>Leann</t>
+  </si>
+  <si>
+    <t>Doyle</t>
+  </si>
+  <si>
+    <t>070-417-641</t>
+  </si>
+  <si>
+    <t>261 Tills</t>
+  </si>
+  <si>
+    <t>Test18</t>
+  </si>
+  <si>
+    <t>10699373</t>
+  </si>
+  <si>
+    <t>Brycen</t>
+  </si>
+  <si>
+    <t>Bode</t>
+  </si>
+  <si>
+    <t>070-417-642</t>
+  </si>
+  <si>
+    <t>25 Primarket</t>
+  </si>
+  <si>
+    <t>Test19</t>
+  </si>
+  <si>
+    <t>10699368</t>
+  </si>
+  <si>
+    <t>Brandy</t>
+  </si>
+  <si>
+    <t>Rath</t>
+  </si>
+  <si>
+    <t>070-417-643</t>
+  </si>
+  <si>
+    <t>260 Fitting Rooms</t>
+  </si>
+  <si>
+    <t>Test20</t>
+  </si>
+  <si>
+    <t>10699372</t>
+  </si>
+  <si>
+    <t>Aurore</t>
+  </si>
+  <si>
+    <t>Grady</t>
+  </si>
+  <si>
+    <t>070-417-644</t>
+  </si>
+  <si>
+    <t>10699341</t>
+  </si>
+  <si>
+    <t>Test failed for 'Fannie Batz' Employee: Errors and AlertsErrorErrorDepartment/Section is required to have a value. &amp; find failed Screenshot Path:-&gt;H:\Clone-Workday-Playwright/WorkdayFailedScreenshot/2025-05-26T11-12-52-966Z.png</t>
+  </si>
+  <si>
+    <t>10699352</t>
+  </si>
+  <si>
+    <t>10699355</t>
+  </si>
+  <si>
+    <t>10699357</t>
+  </si>
+  <si>
+    <t>10699359</t>
+  </si>
+  <si>
+    <t>10699367</t>
+  </si>
+  <si>
+    <t>10699362</t>
   </si>
   <si>
     <t>Failed</t>
-  </si>
-  <si>
-    <t>TestTwentySix</t>
-  </si>
-  <si>
-    <t>070-417-636</t>
-  </si>
-  <si>
-    <t>07 Footwear</t>
-  </si>
-  <si>
-    <t>Test13</t>
-  </si>
-  <si>
-    <t>TestTwentySeven</t>
-  </si>
-  <si>
-    <t>070-417-637</t>
-  </si>
-  <si>
-    <t>08 Ladieswear</t>
-  </si>
-  <si>
-    <t>Test14</t>
-  </si>
-  <si>
-    <t>TestTwentyEight</t>
-  </si>
-  <si>
-    <t>070-417-638</t>
-  </si>
-  <si>
-    <t>6 Days (Slovenia)</t>
-  </si>
-  <si>
-    <t>11 Household</t>
-  </si>
-  <si>
-    <t>Test15</t>
-  </si>
-  <si>
-    <t>TestTwentyNine</t>
-  </si>
-  <si>
-    <t>070-417-639</t>
-  </si>
-  <si>
-    <t>15 Children's Accessories</t>
-  </si>
-  <si>
-    <t>Test16</t>
-  </si>
-  <si>
-    <t>TestThirty</t>
-  </si>
-  <si>
-    <t>070-417-640</t>
-  </si>
-  <si>
-    <t>23 Health &amp; Beauty</t>
-  </si>
-  <si>
-    <t>Test17</t>
-  </si>
-  <si>
-    <t>TestThirtyOne</t>
-  </si>
-  <si>
-    <t>070-417-641</t>
-  </si>
-  <si>
-    <t>261 Tills</t>
-  </si>
-  <si>
-    <t>Test18</t>
-  </si>
-  <si>
-    <t>TestThirtyTwo</t>
-  </si>
-  <si>
-    <t>070-417-642</t>
-  </si>
-  <si>
-    <t>25 Primarket</t>
-  </si>
-  <si>
-    <t>Test19</t>
-  </si>
-  <si>
-    <t>TestThirtyThree</t>
-  </si>
-  <si>
-    <t>070-417-643</t>
-  </si>
-  <si>
-    <t>260 Fitting Rooms</t>
-  </si>
-  <si>
-    <t>Test20</t>
-  </si>
-  <si>
-    <t>TestThirtyFour</t>
-  </si>
-  <si>
-    <t>070-417-644</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="mm/dd/yyyy"/>
   </numFmts>
   <fonts count="8" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-      <sz val="11"/>
-      <name val="Calibri"/>
     </font>
     <font>
+      <sz val="14"/>
       <color rgb="FFFF0000"/>
+      <name val="Arial"/>
       <family val="2"/>
-      <sz val="14"/>
-      <name val="Arial"/>
     </font>
     <font>
+      <sz val="14"/>
       <color theme="1"/>
+      <name val="Arial"/>
       <family val="2"/>
-      <sz val="14"/>
-      <name val="Arial"/>
     </font>
     <font>
       <b/>
+      <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
       <sz val="11"/>
       <name val="Calibri"/>
-    </font>
-    <font>
       <family val="2"/>
       <scheme val="minor"/>
-      <sz val="11"/>
-      <name val="Calibri"/>
     </font>
     <font>
       <u/>
+      <sz val="11"/>
       <color theme="10"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-      <sz val="11"/>
-      <name val="Calibri"/>
     </font>
     <font>
+      <sz val="11"/>
       <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-      <sz val="11"/>
-      <name val="Calibri"/>
     </font>
     <font>
-      <family val="2"/>
       <sz val="14"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -922,19 +773,19 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.5999938962981048"/>
+        <fgColor theme="5" tint="0.59999389629810485"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="0" tint="-0.1499984740745262"/>
+        <fgColor theme="0" tint="-0.14999847407452621"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.7999816888943144"/>
+        <fgColor theme="5" tint="0.79998168889431442"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -947,6 +798,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF00FF00"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF0000"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -965,15 +822,27 @@
       <right style="medium">
         <color indexed="64"/>
       </right>
-      <top style="thin"/>
-      <bottom style="thin"/>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
       <diagonal/>
     </border>
     <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -984,14 +853,16 @@
         <color indexed="64"/>
       </right>
       <top/>
-      <bottom style="thin"/>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
       <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="37">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -1088,6 +959,9 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" wrapText="1"/>
       <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1368,9 +1242,9 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:BV21"/>
-  <sheetFormatPr defaultRowHeight="15.65" outlineLevelRow="1" outlineLevelCol="0" x14ac:dyDescent="0.35" customHeight="1"/>
+  <sheetFormatPr defaultRowHeight="15.65" customHeight="1" outlineLevelRow="1" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="10.81640625" style="1" customWidth="1"/>
     <col min="2" max="2" width="40.54296875" style="1" customWidth="1"/>
@@ -1445,7 +1319,7 @@
     <col min="74" max="74" width="29" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="14.5" customHeight="1" spans="1:74" s="3" customFormat="1" x14ac:dyDescent="0.25" outlineLevel="1" collapsed="1">
+    <row r="1" spans="1:74" s="3" customFormat="1" ht="14.5" customHeight="1" outlineLevel="1" collapsed="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -1669,11 +1543,13 @@
         <v>69</v>
       </c>
     </row>
-    <row r="2" ht="15.65" customHeight="1" spans="1:74" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:74" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="B2" s="10"/>
+      <c r="B2" s="10" t="s">
+        <v>214</v>
+      </c>
       <c r="C2" s="11" t="s">
         <v>71</v>
       </c>
@@ -1699,8 +1575,8 @@
         <v>78</v>
       </c>
       <c r="K2" s="17">
-        <f t="shared" ref="K2:K21" si="0">TODAY()-7</f>
-        <v>45796</v>
+        <f t="shared" ref="K2:K21" ca="1" si="0">TODAY()-7</f>
+        <v>45797</v>
       </c>
       <c r="L2" s="13" t="s">
         <v>73</v>
@@ -1730,8 +1606,8 @@
         <v>78</v>
       </c>
       <c r="U2" s="22">
-        <f>TODAY()-100</f>
-        <v>45703</v>
+        <f ca="1">TODAY()-100</f>
+        <v>45704</v>
       </c>
       <c r="V2" s="16" t="s">
         <v>83</v>
@@ -1776,20 +1652,20 @@
         <v>89</v>
       </c>
       <c r="AJ2" s="17">
-        <f>TODAY()-100</f>
-        <v>45703</v>
+        <f ca="1">TODAY()-100</f>
+        <v>45704</v>
       </c>
       <c r="AK2" s="17">
-        <f t="shared" ref="AK2:AL2" si="1">TODAY()-100</f>
-        <v>45703</v>
+        <f t="shared" ref="AK2:AL2" ca="1" si="1">TODAY()-100</f>
+        <v>45704</v>
       </c>
       <c r="AL2" s="17">
-        <f t="shared" si="1"/>
-        <v>45703</v>
-      </c>
-      <c r="AM2" s="22">
+        <f t="shared" ca="1" si="1"/>
+        <v>45704</v>
+      </c>
+      <c r="AM2" s="22" t="str">
         <f t="shared" ref="AM2:AM3" si="2">AF2</f>
-        <v>NaN</v>
+        <v>N/A</v>
       </c>
       <c r="AN2" s="16">
         <v>92</v>
@@ -1813,8 +1689,8 @@
         <v>89</v>
       </c>
       <c r="AU2" s="17">
-        <f t="shared" ref="AU2:AU21" si="3">TODAY()+7</f>
-        <v>45810</v>
+        <f t="shared" ref="AU2:AU21" ca="1" si="3">TODAY()+7</f>
+        <v>45811</v>
       </c>
       <c r="AV2" s="13" t="s">
         <v>73</v>
@@ -1823,8 +1699,8 @@
         <v>97</v>
       </c>
       <c r="AX2" s="30">
-        <f t="array" ref="AX2:AX3">_xlfn.RANDARRAY(2,1,1023456789000,9999999999999,TRUE)</f>
-        <v>4604024494235</v>
+        <f t="array" aca="1" ref="AX2:AX3" ca="1">_xlfn.RANDARRAY(2,1,1023456789000,9999999999999,TRUE)</f>
+        <v>8839614952846</v>
       </c>
       <c r="AY2" s="17" t="s">
         <v>98</v>
@@ -1839,8 +1715,8 @@
         <v>100</v>
       </c>
       <c r="BC2" s="30">
-        <f t="array" ref="BC2:BC3">_xlfn.RANDARRAY(2,1,12345678,99999999,TRUE)</f>
-        <v>57140963</v>
+        <f t="array" aca="1" ref="BC2:BC3" ca="1">_xlfn.RANDARRAY(2,1,12345678,99999999,TRUE)</f>
+        <v>75710792</v>
       </c>
       <c r="BD2" s="17" t="s">
         <v>98</v>
@@ -1882,8 +1758,8 @@
         <v>108</v>
       </c>
       <c r="BQ2" s="13">
-        <f t="array" ref="BQ2:BQ3">_xlfn.RANDARRAY(2,1,12345,99999,TRUE)</f>
-        <v>86876</v>
+        <f t="array" aca="1" ref="BQ2:BQ3" ca="1">_xlfn.RANDARRAY(2,1,12345,99999,TRUE)</f>
+        <v>61054</v>
       </c>
       <c r="BR2" s="17">
         <v>44562</v>
@@ -1895,20 +1771,22 @@
         <v>44562</v>
       </c>
       <c r="BU2" s="22">
-        <f t="shared" ref="BU2:BU21" si="4">TODAY()+365</f>
-        <v>46168</v>
+        <f t="shared" ref="BU2:BU21" ca="1" si="4">TODAY()+365</f>
+        <v>46169</v>
       </c>
       <c r="BV2" s="16" t="s">
         <v>109</v>
       </c>
     </row>
-    <row r="3" ht="15.65" customHeight="1" spans="1:74" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:74" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
         <v>110</v>
       </c>
-      <c r="B3" s="10"/>
-      <c r="C3" s="11" t="s">
-        <v>71</v>
+      <c r="B3" s="10" t="s">
+        <v>215</v>
+      </c>
+      <c r="C3" s="36" t="s">
+        <v>222</v>
       </c>
       <c r="D3" s="12" t="s">
         <v>111</v>
@@ -1932,8 +1810,8 @@
         <v>78</v>
       </c>
       <c r="K3" s="17">
-        <f t="shared" si="0"/>
-        <v>45796</v>
+        <f t="shared" ca="1" si="0"/>
+        <v>45797</v>
       </c>
       <c r="L3" s="13" t="s">
         <v>73</v>
@@ -1963,8 +1841,8 @@
         <v>78</v>
       </c>
       <c r="U3" s="22">
-        <f>TODAY()-100</f>
-        <v>45703</v>
+        <f ca="1">TODAY()-100</f>
+        <v>45704</v>
       </c>
       <c r="V3" s="16" t="s">
         <v>83</v>
@@ -2009,20 +1887,20 @@
         <v>89</v>
       </c>
       <c r="AJ3" s="17">
-        <f>TODAY()-100</f>
-        <v>45703</v>
+        <f ca="1">TODAY()-100</f>
+        <v>45704</v>
       </c>
       <c r="AK3" s="17">
-        <f t="shared" ref="AK3:AL3" si="5">TODAY()-100</f>
-        <v>45703</v>
+        <f t="shared" ref="AK3:AL3" ca="1" si="5">TODAY()-100</f>
+        <v>45704</v>
       </c>
       <c r="AL3" s="17">
-        <f t="shared" si="5"/>
-        <v>45703</v>
-      </c>
-      <c r="AM3" s="22">
+        <f t="shared" ca="1" si="5"/>
+        <v>45704</v>
+      </c>
+      <c r="AM3" s="22" t="str">
         <f t="shared" si="2"/>
-        <v>NaN</v>
+        <v>N/A</v>
       </c>
       <c r="AN3" s="16" t="s">
         <v>117</v>
@@ -2046,8 +1924,8 @@
         <v>89</v>
       </c>
       <c r="AU3" s="17">
-        <f t="shared" si="3"/>
-        <v>45810</v>
+        <f t="shared" ca="1" si="3"/>
+        <v>45811</v>
       </c>
       <c r="AV3" s="13" t="s">
         <v>73</v>
@@ -2056,7 +1934,8 @@
         <v>97</v>
       </c>
       <c r="AX3" s="30">
-        <v>9493952194343</v>
+        <f ca="1"/>
+        <v>9051408639195</v>
       </c>
       <c r="AY3" s="17" t="s">
         <v>98</v>
@@ -2071,7 +1950,8 @@
         <v>100</v>
       </c>
       <c r="BC3" s="30">
-        <v>89460822</v>
+        <f ca="1"/>
+        <v>71519290</v>
       </c>
       <c r="BD3" s="17" t="s">
         <v>98</v>
@@ -2113,7 +1993,8 @@
         <v>108</v>
       </c>
       <c r="BQ3" s="13">
-        <v>92128</v>
+        <f ca="1"/>
+        <v>64418</v>
       </c>
       <c r="BR3" s="17">
         <v>44562</v>
@@ -2125,18 +2006,20 @@
         <v>44562</v>
       </c>
       <c r="BU3" s="22">
-        <f t="shared" si="4"/>
-        <v>46168</v>
+        <f t="shared" ca="1" si="4"/>
+        <v>46169</v>
       </c>
       <c r="BV3" s="16" t="s">
         <v>109</v>
       </c>
     </row>
-    <row r="4" ht="15.65" customHeight="1" spans="1:74" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:74" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="B4" s="10"/>
+      <c r="B4" s="10" t="s">
+        <v>216</v>
+      </c>
       <c r="C4" s="11" t="s">
         <v>71</v>
       </c>
@@ -2162,8 +2045,8 @@
         <v>78</v>
       </c>
       <c r="K4" s="17">
-        <f t="shared" si="0"/>
-        <v>45796</v>
+        <f t="shared" ca="1" si="0"/>
+        <v>45797</v>
       </c>
       <c r="L4" s="13" t="s">
         <v>73</v>
@@ -2193,8 +2076,8 @@
         <v>78</v>
       </c>
       <c r="U4" s="22">
-        <f t="shared" ref="U4:U21" si="6">TODAY()-100</f>
-        <v>45703</v>
+        <f t="shared" ref="U4:U21" ca="1" si="6">TODAY()-100</f>
+        <v>45704</v>
       </c>
       <c r="V4" s="16" t="s">
         <v>83</v>
@@ -2239,20 +2122,20 @@
         <v>89</v>
       </c>
       <c r="AJ4" s="17">
-        <f t="shared" ref="AJ4:AL21" si="7">TODAY()-100</f>
-        <v>45703</v>
+        <f t="shared" ref="AJ4:AL21" ca="1" si="7">TODAY()-100</f>
+        <v>45704</v>
       </c>
       <c r="AK4" s="17">
-        <f t="shared" si="7"/>
-        <v>45703</v>
+        <f t="shared" ca="1" si="7"/>
+        <v>45704</v>
       </c>
       <c r="AL4" s="17">
-        <f t="shared" si="7"/>
-        <v>45703</v>
-      </c>
-      <c r="AM4" s="22">
+        <f t="shared" ca="1" si="7"/>
+        <v>45704</v>
+      </c>
+      <c r="AM4" s="22" t="str">
         <f t="shared" ref="AM4:AM6" si="8">AF4</f>
-        <v>NaN</v>
+        <v>N/A</v>
       </c>
       <c r="AN4" s="16" t="s">
         <v>117</v>
@@ -2276,8 +2159,8 @@
         <v>89</v>
       </c>
       <c r="AU4" s="17">
-        <f t="shared" si="3"/>
-        <v>45810</v>
+        <f t="shared" ca="1" si="3"/>
+        <v>45811</v>
       </c>
       <c r="AV4" s="13" t="s">
         <v>73</v>
@@ -2286,8 +2169,8 @@
         <v>97</v>
       </c>
       <c r="AX4" s="30">
-        <f t="array" ref="AX4">_xlfn.RANDARRAY(2,1,1023456789000,9999999999999,TRUE)</f>
-        <v>1391537902519</v>
+        <f t="array" aca="1" ref="AX4" ca="1">_xlfn.RANDARRAY(2,1,1023456789000,9999999999999,TRUE)</f>
+        <v>9274143631434</v>
       </c>
       <c r="AY4" s="17" t="s">
         <v>98</v>
@@ -2302,8 +2185,8 @@
         <v>100</v>
       </c>
       <c r="BC4" s="30">
-        <f t="array" ref="BC4">_xlfn.RANDARRAY(2,1,12345678,99999999,TRUE)</f>
-        <v>98733475</v>
+        <f t="array" aca="1" ref="BC4" ca="1">_xlfn.RANDARRAY(2,1,12345678,99999999,TRUE)</f>
+        <v>88076371</v>
       </c>
       <c r="BD4" s="17" t="s">
         <v>98</v>
@@ -2345,8 +2228,8 @@
         <v>108</v>
       </c>
       <c r="BQ4" s="13">
-        <f t="array" ref="BQ4">_xlfn.RANDARRAY(2,1,12345,99999,TRUE)</f>
-        <v>14778</v>
+        <f t="array" aca="1" ref="BQ4" ca="1">_xlfn.RANDARRAY(2,1,12345,99999,TRUE)</f>
+        <v>13645</v>
       </c>
       <c r="BR4" s="17">
         <v>44562</v>
@@ -2358,18 +2241,20 @@
         <v>44562</v>
       </c>
       <c r="BU4" s="22">
-        <f t="shared" si="4"/>
-        <v>46168</v>
+        <f t="shared" ca="1" si="4"/>
+        <v>46169</v>
       </c>
       <c r="BV4" s="16" t="s">
         <v>109</v>
       </c>
     </row>
-    <row r="5" ht="15.65" customHeight="1" spans="1:74" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:74" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
         <v>123</v>
       </c>
-      <c r="B5" s="10"/>
+      <c r="B5" s="10" t="s">
+        <v>217</v>
+      </c>
       <c r="C5" s="11" t="s">
         <v>71</v>
       </c>
@@ -2395,8 +2280,8 @@
         <v>78</v>
       </c>
       <c r="K5" s="17">
-        <f t="shared" si="0"/>
-        <v>45796</v>
+        <f t="shared" ca="1" si="0"/>
+        <v>45797</v>
       </c>
       <c r="L5" s="13" t="s">
         <v>73</v>
@@ -2426,8 +2311,8 @@
         <v>78</v>
       </c>
       <c r="U5" s="22">
-        <f t="shared" si="6"/>
-        <v>45703</v>
+        <f t="shared" ca="1" si="6"/>
+        <v>45704</v>
       </c>
       <c r="V5" s="16" t="s">
         <v>83</v>
@@ -2472,20 +2357,20 @@
         <v>89</v>
       </c>
       <c r="AJ5" s="17">
-        <f t="shared" si="7"/>
-        <v>45703</v>
+        <f t="shared" ca="1" si="7"/>
+        <v>45704</v>
       </c>
       <c r="AK5" s="17">
-        <f t="shared" si="7"/>
-        <v>45703</v>
+        <f t="shared" ca="1" si="7"/>
+        <v>45704</v>
       </c>
       <c r="AL5" s="17">
-        <f t="shared" si="7"/>
-        <v>45703</v>
-      </c>
-      <c r="AM5" s="22">
+        <f t="shared" ca="1" si="7"/>
+        <v>45704</v>
+      </c>
+      <c r="AM5" s="22" t="str">
         <f t="shared" si="8"/>
-        <v>NaN</v>
+        <v>N/A</v>
       </c>
       <c r="AN5" s="16" t="s">
         <v>117</v>
@@ -2509,8 +2394,8 @@
         <v>89</v>
       </c>
       <c r="AU5" s="17">
-        <f t="shared" si="3"/>
-        <v>45810</v>
+        <f t="shared" ca="1" si="3"/>
+        <v>45811</v>
       </c>
       <c r="AV5" s="13" t="s">
         <v>73</v>
@@ -2519,8 +2404,8 @@
         <v>97</v>
       </c>
       <c r="AX5" s="30">
-        <f t="array" ref="AX5">_xlfn.RANDARRAY(2,1,1023456789000,9999999999999,TRUE)</f>
-        <v>9919835811153</v>
+        <f t="array" aca="1" ref="AX5" ca="1">_xlfn.RANDARRAY(2,1,1023456789000,9999999999999,TRUE)</f>
+        <v>5139643126152</v>
       </c>
       <c r="AY5" s="17" t="s">
         <v>98</v>
@@ -2535,8 +2420,8 @@
         <v>100</v>
       </c>
       <c r="BC5" s="30">
-        <f t="array" ref="BC5">_xlfn.RANDARRAY(2,1,12345678,99999999,TRUE)</f>
-        <v>52371519</v>
+        <f t="array" aca="1" ref="BC5" ca="1">_xlfn.RANDARRAY(2,1,12345678,99999999,TRUE)</f>
+        <v>12634481</v>
       </c>
       <c r="BD5" s="17" t="s">
         <v>98</v>
@@ -2578,8 +2463,8 @@
         <v>108</v>
       </c>
       <c r="BQ5" s="13">
-        <f t="array" ref="BQ5">_xlfn.RANDARRAY(2,1,12345,99999,TRUE)</f>
-        <v>33930</v>
+        <f t="array" aca="1" ref="BQ5" ca="1">_xlfn.RANDARRAY(2,1,12345,99999,TRUE)</f>
+        <v>82087</v>
       </c>
       <c r="BR5" s="17">
         <v>44562</v>
@@ -2591,18 +2476,20 @@
         <v>44562</v>
       </c>
       <c r="BU5" s="22">
-        <f t="shared" si="4"/>
-        <v>46168</v>
+        <f t="shared" ca="1" si="4"/>
+        <v>46169</v>
       </c>
       <c r="BV5" s="16" t="s">
         <v>109</v>
       </c>
     </row>
-    <row r="6" ht="15.65" customHeight="1" spans="1:74" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:74" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
         <v>127</v>
       </c>
-      <c r="B6" s="10"/>
+      <c r="B6" s="10" t="s">
+        <v>218</v>
+      </c>
       <c r="C6" s="11" t="s">
         <v>71</v>
       </c>
@@ -2628,8 +2515,8 @@
         <v>78</v>
       </c>
       <c r="K6" s="17">
-        <f t="shared" si="0"/>
-        <v>45796</v>
+        <f t="shared" ca="1" si="0"/>
+        <v>45797</v>
       </c>
       <c r="L6" s="13" t="s">
         <v>73</v>
@@ -2659,8 +2546,8 @@
         <v>78</v>
       </c>
       <c r="U6" s="22">
-        <f t="shared" si="6"/>
-        <v>45703</v>
+        <f t="shared" ca="1" si="6"/>
+        <v>45704</v>
       </c>
       <c r="V6" s="16" t="s">
         <v>83</v>
@@ -2705,20 +2592,20 @@
         <v>89</v>
       </c>
       <c r="AJ6" s="17">
-        <f t="shared" si="7"/>
-        <v>45703</v>
+        <f t="shared" ca="1" si="7"/>
+        <v>45704</v>
       </c>
       <c r="AK6" s="17">
-        <f t="shared" si="7"/>
-        <v>45703</v>
+        <f t="shared" ca="1" si="7"/>
+        <v>45704</v>
       </c>
       <c r="AL6" s="17">
-        <f t="shared" si="7"/>
-        <v>45703</v>
-      </c>
-      <c r="AM6" s="22">
+        <f t="shared" ca="1" si="7"/>
+        <v>45704</v>
+      </c>
+      <c r="AM6" s="22" t="str">
         <f t="shared" si="8"/>
-        <v>NaN</v>
+        <v>N/A</v>
       </c>
       <c r="AN6" s="16" t="s">
         <v>117</v>
@@ -2742,8 +2629,8 @@
         <v>89</v>
       </c>
       <c r="AU6" s="17">
-        <f t="shared" si="3"/>
-        <v>45810</v>
+        <f t="shared" ca="1" si="3"/>
+        <v>45811</v>
       </c>
       <c r="AV6" s="13" t="s">
         <v>73</v>
@@ -2752,8 +2639,8 @@
         <v>97</v>
       </c>
       <c r="AX6" s="30">
-        <f t="array" ref="AX6">_xlfn.RANDARRAY(2,1,1023456789000,9999999999999,TRUE)</f>
-        <v>5828963909979</v>
+        <f t="array" aca="1" ref="AX6" ca="1">_xlfn.RANDARRAY(2,1,1023456789000,9999999999999,TRUE)</f>
+        <v>3243945052231</v>
       </c>
       <c r="AY6" s="17" t="s">
         <v>98</v>
@@ -2768,8 +2655,8 @@
         <v>100</v>
       </c>
       <c r="BC6" s="30">
-        <f t="array" ref="BC6">_xlfn.RANDARRAY(2,1,12345678,99999999,TRUE)</f>
-        <v>62669539</v>
+        <f t="array" aca="1" ref="BC6" ca="1">_xlfn.RANDARRAY(2,1,12345678,99999999,TRUE)</f>
+        <v>50022118</v>
       </c>
       <c r="BD6" s="17" t="s">
         <v>98</v>
@@ -2811,8 +2698,8 @@
         <v>108</v>
       </c>
       <c r="BQ6" s="13">
-        <f t="array" ref="BQ6">_xlfn.RANDARRAY(2,1,12345,99999,TRUE)</f>
-        <v>43725</v>
+        <f t="array" aca="1" ref="BQ6" ca="1">_xlfn.RANDARRAY(2,1,12345,99999,TRUE)</f>
+        <v>55453</v>
       </c>
       <c r="BR6" s="17">
         <v>44562</v>
@@ -2824,18 +2711,20 @@
         <v>44562</v>
       </c>
       <c r="BU6" s="22">
-        <f t="shared" si="4"/>
-        <v>46168</v>
+        <f t="shared" ca="1" si="4"/>
+        <v>46169</v>
       </c>
       <c r="BV6" s="16" t="s">
         <v>109</v>
       </c>
     </row>
-    <row r="7" ht="15.65" customHeight="1" spans="1:74" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:74" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
         <v>132</v>
       </c>
-      <c r="B7" s="10"/>
+      <c r="B7" s="10" t="s">
+        <v>219</v>
+      </c>
       <c r="C7" s="11" t="s">
         <v>71</v>
       </c>
@@ -2861,8 +2750,8 @@
         <v>78</v>
       </c>
       <c r="K7" s="17">
-        <f t="shared" si="0"/>
-        <v>45796</v>
+        <f t="shared" ca="1" si="0"/>
+        <v>45797</v>
       </c>
       <c r="L7" s="13" t="s">
         <v>73</v>
@@ -2892,8 +2781,8 @@
         <v>78</v>
       </c>
       <c r="U7" s="22">
-        <f t="shared" si="6"/>
-        <v>45703</v>
+        <f t="shared" ca="1" si="6"/>
+        <v>45704</v>
       </c>
       <c r="V7" s="16" t="s">
         <v>83</v>
@@ -2938,20 +2827,20 @@
         <v>89</v>
       </c>
       <c r="AJ7" s="17">
-        <f t="shared" si="7"/>
-        <v>45703</v>
+        <f t="shared" ca="1" si="7"/>
+        <v>45704</v>
       </c>
       <c r="AK7" s="17">
-        <f t="shared" si="7"/>
-        <v>45703</v>
+        <f t="shared" ca="1" si="7"/>
+        <v>45704</v>
       </c>
       <c r="AL7" s="17">
-        <f t="shared" si="7"/>
-        <v>45703</v>
-      </c>
-      <c r="AM7" s="22">
+        <f t="shared" ca="1" si="7"/>
+        <v>45704</v>
+      </c>
+      <c r="AM7" s="22" t="str">
         <f t="shared" ref="AM7:AM9" si="9">AF7</f>
-        <v>NaN</v>
+        <v>N/A</v>
       </c>
       <c r="AN7" s="16" t="s">
         <v>117</v>
@@ -2975,8 +2864,8 @@
         <v>89</v>
       </c>
       <c r="AU7" s="17">
-        <f t="shared" si="3"/>
-        <v>45810</v>
+        <f t="shared" ca="1" si="3"/>
+        <v>45811</v>
       </c>
       <c r="AV7" s="13" t="s">
         <v>73</v>
@@ -2985,8 +2874,8 @@
         <v>97</v>
       </c>
       <c r="AX7" s="30">
-        <f t="array" ref="AX7">_xlfn.RANDARRAY(2,1,1023456789000,9999999999999,TRUE)</f>
-        <v>3023536623629</v>
+        <f t="array" aca="1" ref="AX7" ca="1">_xlfn.RANDARRAY(2,1,1023456789000,9999999999999,TRUE)</f>
+        <v>7664329445131</v>
       </c>
       <c r="AY7" s="17" t="s">
         <v>98</v>
@@ -3001,8 +2890,8 @@
         <v>100</v>
       </c>
       <c r="BC7" s="30">
-        <f t="array" ref="BC7">_xlfn.RANDARRAY(2,1,12345678,99999999,TRUE)</f>
-        <v>90682523</v>
+        <f t="array" aca="1" ref="BC7" ca="1">_xlfn.RANDARRAY(2,1,12345678,99999999,TRUE)</f>
+        <v>33676766</v>
       </c>
       <c r="BD7" s="17" t="s">
         <v>98</v>
@@ -3044,8 +2933,8 @@
         <v>108</v>
       </c>
       <c r="BQ7" s="13">
-        <f t="array" ref="BQ7">_xlfn.RANDARRAY(2,1,12345,99999,TRUE)</f>
-        <v>70827</v>
+        <f t="array" aca="1" ref="BQ7" ca="1">_xlfn.RANDARRAY(2,1,12345,99999,TRUE)</f>
+        <v>39708</v>
       </c>
       <c r="BR7" s="17">
         <v>44562</v>
@@ -3057,18 +2946,20 @@
         <v>44562</v>
       </c>
       <c r="BU7" s="22">
-        <f t="shared" si="4"/>
-        <v>46168</v>
+        <f t="shared" ca="1" si="4"/>
+        <v>46169</v>
       </c>
       <c r="BV7" s="16" t="s">
         <v>109</v>
       </c>
     </row>
-    <row r="8" ht="15.65" customHeight="1" spans="1:74" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:74" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="1" t="s">
         <v>135</v>
       </c>
-      <c r="B8" s="10"/>
+      <c r="B8" s="10" t="s">
+        <v>220</v>
+      </c>
       <c r="C8" s="11" t="s">
         <v>71</v>
       </c>
@@ -3094,8 +2985,8 @@
         <v>78</v>
       </c>
       <c r="K8" s="17">
-        <f t="shared" si="0"/>
-        <v>45796</v>
+        <f t="shared" ca="1" si="0"/>
+        <v>45797</v>
       </c>
       <c r="L8" s="13" t="s">
         <v>73</v>
@@ -3125,8 +3016,8 @@
         <v>78</v>
       </c>
       <c r="U8" s="22">
-        <f t="shared" si="6"/>
-        <v>45703</v>
+        <f t="shared" ca="1" si="6"/>
+        <v>45704</v>
       </c>
       <c r="V8" s="16" t="s">
         <v>83</v>
@@ -3171,20 +3062,20 @@
         <v>89</v>
       </c>
       <c r="AJ8" s="17">
-        <f t="shared" si="7"/>
-        <v>45703</v>
+        <f t="shared" ca="1" si="7"/>
+        <v>45704</v>
       </c>
       <c r="AK8" s="17">
-        <f t="shared" si="7"/>
-        <v>45703</v>
+        <f t="shared" ca="1" si="7"/>
+        <v>45704</v>
       </c>
       <c r="AL8" s="17">
-        <f t="shared" si="7"/>
-        <v>45703</v>
-      </c>
-      <c r="AM8" s="22">
+        <f t="shared" ca="1" si="7"/>
+        <v>45704</v>
+      </c>
+      <c r="AM8" s="22" t="str">
         <f t="shared" si="9"/>
-        <v>NaN</v>
+        <v>N/A</v>
       </c>
       <c r="AN8" s="16" t="s">
         <v>117</v>
@@ -3208,8 +3099,8 @@
         <v>89</v>
       </c>
       <c r="AU8" s="17">
-        <f t="shared" si="3"/>
-        <v>45810</v>
+        <f t="shared" ca="1" si="3"/>
+        <v>45811</v>
       </c>
       <c r="AV8" s="13" t="s">
         <v>73</v>
@@ -3218,8 +3109,8 @@
         <v>97</v>
       </c>
       <c r="AX8" s="30">
-        <f t="array" ref="AX8">_xlfn.RANDARRAY(2,1,1023456789000,9999999999999,TRUE)</f>
-        <v>8032780328091</v>
+        <f t="array" aca="1" ref="AX8" ca="1">_xlfn.RANDARRAY(2,1,1023456789000,9999999999999,TRUE)</f>
+        <v>4251987508942</v>
       </c>
       <c r="AY8" s="17" t="s">
         <v>98</v>
@@ -3234,8 +3125,8 @@
         <v>100</v>
       </c>
       <c r="BC8" s="30">
-        <f t="array" ref="BC8">_xlfn.RANDARRAY(2,1,12345678,99999999,TRUE)</f>
-        <v>52624529</v>
+        <f t="array" aca="1" ref="BC8" ca="1">_xlfn.RANDARRAY(2,1,12345678,99999999,TRUE)</f>
+        <v>74202321</v>
       </c>
       <c r="BD8" s="17" t="s">
         <v>98</v>
@@ -3277,8 +3168,8 @@
         <v>108</v>
       </c>
       <c r="BQ8" s="13">
-        <f t="array" ref="BQ8">_xlfn.RANDARRAY(2,1,12345,99999,TRUE)</f>
-        <v>46031</v>
+        <f t="array" aca="1" ref="BQ8" ca="1">_xlfn.RANDARRAY(2,1,12345,99999,TRUE)</f>
+        <v>28796</v>
       </c>
       <c r="BR8" s="17">
         <v>44562</v>
@@ -3290,18 +3181,20 @@
         <v>44562</v>
       </c>
       <c r="BU8" s="22">
-        <f t="shared" si="4"/>
-        <v>46168</v>
+        <f t="shared" ca="1" si="4"/>
+        <v>46169</v>
       </c>
       <c r="BV8" s="16" t="s">
         <v>109</v>
       </c>
     </row>
-    <row r="9" ht="15.65" customHeight="1" spans="1:74" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:74" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="1" t="s">
         <v>138</v>
       </c>
-      <c r="B9" s="10"/>
+      <c r="B9" s="10" t="s">
+        <v>221</v>
+      </c>
       <c r="C9" s="11" t="s">
         <v>71</v>
       </c>
@@ -3327,8 +3220,8 @@
         <v>78</v>
       </c>
       <c r="K9" s="17">
-        <f t="shared" si="0"/>
-        <v>45796</v>
+        <f t="shared" ca="1" si="0"/>
+        <v>45797</v>
       </c>
       <c r="L9" s="13" t="s">
         <v>73</v>
@@ -3358,8 +3251,8 @@
         <v>78</v>
       </c>
       <c r="U9" s="22">
-        <f t="shared" si="6"/>
-        <v>45703</v>
+        <f t="shared" ca="1" si="6"/>
+        <v>45704</v>
       </c>
       <c r="V9" s="16" t="s">
         <v>83</v>
@@ -3404,20 +3297,20 @@
         <v>89</v>
       </c>
       <c r="AJ9" s="17">
-        <f t="shared" si="7"/>
-        <v>45703</v>
+        <f t="shared" ca="1" si="7"/>
+        <v>45704</v>
       </c>
       <c r="AK9" s="17">
-        <f t="shared" si="7"/>
-        <v>45703</v>
+        <f t="shared" ca="1" si="7"/>
+        <v>45704</v>
       </c>
       <c r="AL9" s="17">
-        <f t="shared" si="7"/>
-        <v>45703</v>
-      </c>
-      <c r="AM9" s="22">
+        <f t="shared" ca="1" si="7"/>
+        <v>45704</v>
+      </c>
+      <c r="AM9" s="22" t="str">
         <f t="shared" si="9"/>
-        <v>NaN</v>
+        <v>N/A</v>
       </c>
       <c r="AN9" s="16" t="s">
         <v>117</v>
@@ -3441,8 +3334,8 @@
         <v>89</v>
       </c>
       <c r="AU9" s="17">
-        <f t="shared" si="3"/>
-        <v>45810</v>
+        <f t="shared" ca="1" si="3"/>
+        <v>45811</v>
       </c>
       <c r="AV9" s="13" t="s">
         <v>73</v>
@@ -3451,8 +3344,8 @@
         <v>97</v>
       </c>
       <c r="AX9" s="30">
-        <f t="array" ref="AX9">_xlfn.RANDARRAY(2,1,1023456789000,9999999999999,TRUE)</f>
-        <v>8366552217454</v>
+        <f t="array" aca="1" ref="AX9" ca="1">_xlfn.RANDARRAY(2,1,1023456789000,9999999999999,TRUE)</f>
+        <v>5274896221277</v>
       </c>
       <c r="AY9" s="17" t="s">
         <v>98</v>
@@ -3467,8 +3360,8 @@
         <v>100</v>
       </c>
       <c r="BC9" s="30">
-        <f t="array" ref="BC9">_xlfn.RANDARRAY(2,1,12345678,99999999,TRUE)</f>
-        <v>34816810</v>
+        <f t="array" aca="1" ref="BC9" ca="1">_xlfn.RANDARRAY(2,1,12345678,99999999,TRUE)</f>
+        <v>15535144</v>
       </c>
       <c r="BD9" s="17" t="s">
         <v>98</v>
@@ -3510,8 +3403,8 @@
         <v>108</v>
       </c>
       <c r="BQ9" s="13">
-        <f t="array" ref="BQ9">_xlfn.RANDARRAY(2,1,12345,99999,TRUE)</f>
-        <v>24667</v>
+        <f t="array" aca="1" ref="BQ9" ca="1">_xlfn.RANDARRAY(2,1,12345,99999,TRUE)</f>
+        <v>79884</v>
       </c>
       <c r="BR9" s="17">
         <v>44562</v>
@@ -3523,14 +3416,14 @@
         <v>44562</v>
       </c>
       <c r="BU9" s="22">
-        <f t="shared" si="4"/>
-        <v>46168</v>
+        <f t="shared" ca="1" si="4"/>
+        <v>46169</v>
       </c>
       <c r="BV9" s="16" t="s">
         <v>109</v>
       </c>
     </row>
-    <row r="10" ht="15.65" customHeight="1" spans="1:74" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:74" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" s="1" t="s">
         <v>143</v>
       </c>
@@ -3562,8 +3455,8 @@
         <v>78</v>
       </c>
       <c r="K10" s="17">
-        <f t="shared" si="0"/>
-        <v>45796</v>
+        <f t="shared" ca="1" si="0"/>
+        <v>45797</v>
       </c>
       <c r="L10" s="13" t="s">
         <v>73</v>
@@ -3593,8 +3486,8 @@
         <v>78</v>
       </c>
       <c r="U10" s="22">
-        <f t="shared" si="6"/>
-        <v>45703</v>
+        <f t="shared" ca="1" si="6"/>
+        <v>45704</v>
       </c>
       <c r="V10" s="16" t="s">
         <v>83</v>
@@ -3639,20 +3532,20 @@
         <v>89</v>
       </c>
       <c r="AJ10" s="17">
-        <f t="shared" si="7"/>
-        <v>45703</v>
+        <f t="shared" ca="1" si="7"/>
+        <v>45704</v>
       </c>
       <c r="AK10" s="17">
-        <f t="shared" si="7"/>
-        <v>45703</v>
+        <f t="shared" ca="1" si="7"/>
+        <v>45704</v>
       </c>
       <c r="AL10" s="17">
-        <f t="shared" si="7"/>
-        <v>45703</v>
-      </c>
-      <c r="AM10" s="22">
+        <f t="shared" ca="1" si="7"/>
+        <v>45704</v>
+      </c>
+      <c r="AM10" s="22" t="str">
         <f t="shared" ref="AM10:AM13" si="10">AF10</f>
-        <v>NaN</v>
+        <v>N/A</v>
       </c>
       <c r="AN10" s="16" t="s">
         <v>117</v>
@@ -3676,8 +3569,8 @@
         <v>89</v>
       </c>
       <c r="AU10" s="17">
-        <f t="shared" si="3"/>
-        <v>45810</v>
+        <f t="shared" ca="1" si="3"/>
+        <v>45811</v>
       </c>
       <c r="AV10" s="13" t="s">
         <v>73</v>
@@ -3686,8 +3579,8 @@
         <v>97</v>
       </c>
       <c r="AX10" s="30">
-        <f t="array" ref="AX10">_xlfn.RANDARRAY(2,1,1023456789000,9999999999999,TRUE)</f>
-        <v>6642334879451</v>
+        <f t="array" aca="1" ref="AX10" ca="1">_xlfn.RANDARRAY(2,1,1023456789000,9999999999999,TRUE)</f>
+        <v>4946483063267</v>
       </c>
       <c r="AY10" s="17" t="s">
         <v>98</v>
@@ -3702,8 +3595,8 @@
         <v>100</v>
       </c>
       <c r="BC10" s="30">
-        <f t="array" ref="BC10">_xlfn.RANDARRAY(2,1,12345678,99999999,TRUE)</f>
-        <v>38185096</v>
+        <f t="array" aca="1" ref="BC10" ca="1">_xlfn.RANDARRAY(2,1,12345678,99999999,TRUE)</f>
+        <v>74053525</v>
       </c>
       <c r="BD10" s="17" t="s">
         <v>98</v>
@@ -3745,8 +3638,8 @@
         <v>108</v>
       </c>
       <c r="BQ10" s="13">
-        <f t="array" ref="BQ10">_xlfn.RANDARRAY(2,1,12345,99999,TRUE)</f>
-        <v>24793</v>
+        <f t="array" aca="1" ref="BQ10" ca="1">_xlfn.RANDARRAY(2,1,12345,99999,TRUE)</f>
+        <v>34594</v>
       </c>
       <c r="BR10" s="17">
         <v>44562</v>
@@ -3758,19 +3651,23 @@
         <v>44562</v>
       </c>
       <c r="BU10" s="22">
-        <f t="shared" si="4"/>
-        <v>46168</v>
+        <f t="shared" ca="1" si="4"/>
+        <v>46169</v>
       </c>
       <c r="BV10" s="16" t="s">
         <v>109</v>
       </c>
     </row>
-    <row r="11" ht="15.65" customHeight="1" spans="1:74" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:74" ht="15.65" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
         <v>149</v>
       </c>
-      <c r="B11" s="10"/>
-      <c r="C11" s="11"/>
+      <c r="B11" s="10">
+        <v>10699351</v>
+      </c>
+      <c r="C11" s="11" t="s">
+        <v>71</v>
+      </c>
       <c r="D11" s="12" t="s">
         <v>111</v>
       </c>
@@ -3793,8 +3690,8 @@
         <v>78</v>
       </c>
       <c r="K11" s="17">
-        <f t="shared" si="0"/>
-        <v>45796</v>
+        <f t="shared" ca="1" si="0"/>
+        <v>45797</v>
       </c>
       <c r="L11" s="13" t="s">
         <v>73</v>
@@ -3824,8 +3721,8 @@
         <v>78</v>
       </c>
       <c r="U11" s="22">
-        <f t="shared" si="6"/>
-        <v>45703</v>
+        <f t="shared" ca="1" si="6"/>
+        <v>45704</v>
       </c>
       <c r="V11" s="16" t="s">
         <v>83</v>
@@ -3870,20 +3767,20 @@
         <v>89</v>
       </c>
       <c r="AJ11" s="17">
-        <f t="shared" si="7"/>
-        <v>45703</v>
+        <f t="shared" ca="1" si="7"/>
+        <v>45704</v>
       </c>
       <c r="AK11" s="17">
-        <f t="shared" si="7"/>
-        <v>45703</v>
+        <f t="shared" ca="1" si="7"/>
+        <v>45704</v>
       </c>
       <c r="AL11" s="17">
-        <f t="shared" si="7"/>
-        <v>45703</v>
-      </c>
-      <c r="AM11" s="22">
+        <f t="shared" ca="1" si="7"/>
+        <v>45704</v>
+      </c>
+      <c r="AM11" s="22" t="str">
         <f t="shared" si="10"/>
-        <v>NaN</v>
+        <v>N/A</v>
       </c>
       <c r="AN11" s="16" t="s">
         <v>117</v>
@@ -3907,8 +3804,8 @@
         <v>89</v>
       </c>
       <c r="AU11" s="17">
-        <f t="shared" si="3"/>
-        <v>45810</v>
+        <f t="shared" ca="1" si="3"/>
+        <v>45811</v>
       </c>
       <c r="AV11" s="13" t="s">
         <v>73</v>
@@ -3917,8 +3814,8 @@
         <v>97</v>
       </c>
       <c r="AX11" s="30">
-        <f t="array" ref="AX11">_xlfn.RANDARRAY(2,1,1023456789000,9999999999999,TRUE)</f>
-        <v>9842151148722</v>
+        <f t="array" aca="1" ref="AX11" ca="1">_xlfn.RANDARRAY(2,1,1023456789000,9999999999999,TRUE)</f>
+        <v>1730931821023</v>
       </c>
       <c r="AY11" s="17" t="s">
         <v>98</v>
@@ -3933,8 +3830,8 @@
         <v>100</v>
       </c>
       <c r="BC11" s="30">
-        <f t="array" ref="BC11">_xlfn.RANDARRAY(2,1,12345678,99999999,TRUE)</f>
-        <v>93304189</v>
+        <f t="array" aca="1" ref="BC11" ca="1">_xlfn.RANDARRAY(2,1,12345678,99999999,TRUE)</f>
+        <v>46158742</v>
       </c>
       <c r="BD11" s="17" t="s">
         <v>98</v>
@@ -3976,8 +3873,8 @@
         <v>108</v>
       </c>
       <c r="BQ11" s="13">
-        <f t="array" ref="BQ11">_xlfn.RANDARRAY(2,1,12345,99999,TRUE)</f>
-        <v>37705</v>
+        <f t="array" aca="1" ref="BQ11" ca="1">_xlfn.RANDARRAY(2,1,12345,99999,TRUE)</f>
+        <v>38054</v>
       </c>
       <c r="BR11" s="17">
         <v>44562</v>
@@ -3989,19 +3886,23 @@
         <v>44562</v>
       </c>
       <c r="BU11" s="22">
-        <f t="shared" si="4"/>
-        <v>46168</v>
+        <f t="shared" ca="1" si="4"/>
+        <v>46169</v>
       </c>
       <c r="BV11" s="16" t="s">
         <v>109</v>
       </c>
     </row>
-    <row r="12" ht="15.65" customHeight="1" spans="1:74" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:74" ht="15.65" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
         <v>154</v>
       </c>
-      <c r="B12" s="10"/>
-      <c r="C12" s="11"/>
+      <c r="B12" s="10" t="s">
+        <v>155</v>
+      </c>
+      <c r="C12" s="11" t="s">
+        <v>71</v>
+      </c>
       <c r="D12" s="12" t="s">
         <v>111</v>
       </c>
@@ -4009,13 +3910,13 @@
         <v>73</v>
       </c>
       <c r="F12" s="14" t="s">
-        <v>74</v>
+        <v>156</v>
       </c>
       <c r="G12" s="14" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="H12" s="15" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="I12" s="16" t="s">
         <v>77</v>
@@ -4024,8 +3925,8 @@
         <v>78</v>
       </c>
       <c r="K12" s="17">
-        <f t="shared" si="0"/>
-        <v>45796</v>
+        <f t="shared" ca="1" si="0"/>
+        <v>45797</v>
       </c>
       <c r="L12" s="13" t="s">
         <v>73</v>
@@ -4055,8 +3956,8 @@
         <v>78</v>
       </c>
       <c r="U12" s="22">
-        <f t="shared" si="6"/>
-        <v>45703</v>
+        <f t="shared" ca="1" si="6"/>
+        <v>45704</v>
       </c>
       <c r="V12" s="16" t="s">
         <v>83</v>
@@ -4086,7 +3987,7 @@
         <v>89</v>
       </c>
       <c r="AE12" s="33" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="AF12" s="28" t="s">
         <v>89</v>
@@ -4101,26 +4002,26 @@
         <v>89</v>
       </c>
       <c r="AJ12" s="17">
-        <f t="shared" si="7"/>
-        <v>45703</v>
+        <f t="shared" ca="1" si="7"/>
+        <v>45704</v>
       </c>
       <c r="AK12" s="17">
-        <f t="shared" si="7"/>
-        <v>45703</v>
+        <f t="shared" ca="1" si="7"/>
+        <v>45704</v>
       </c>
       <c r="AL12" s="17">
-        <f t="shared" si="7"/>
-        <v>45703</v>
-      </c>
-      <c r="AM12" s="22">
+        <f t="shared" ca="1" si="7"/>
+        <v>45704</v>
+      </c>
+      <c r="AM12" s="22" t="str">
         <f t="shared" si="10"/>
-        <v>NaN</v>
+        <v>N/A</v>
       </c>
       <c r="AN12" s="16" t="s">
         <v>117</v>
       </c>
       <c r="AO12" s="34" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="AP12" s="24" t="s">
         <v>94</v>
@@ -4138,8 +4039,8 @@
         <v>89</v>
       </c>
       <c r="AU12" s="17">
-        <f t="shared" si="3"/>
-        <v>45810</v>
+        <f t="shared" ca="1" si="3"/>
+        <v>45811</v>
       </c>
       <c r="AV12" s="13" t="s">
         <v>73</v>
@@ -4148,8 +4049,8 @@
         <v>97</v>
       </c>
       <c r="AX12" s="30">
-        <f t="array" ref="AX12">_xlfn.RANDARRAY(2,1,1023456789000,9999999999999,TRUE)</f>
-        <v>4729294405842</v>
+        <f t="array" aca="1" ref="AX12" ca="1">_xlfn.RANDARRAY(2,1,1023456789000,9999999999999,TRUE)</f>
+        <v>1667026353095</v>
       </c>
       <c r="AY12" s="17" t="s">
         <v>98</v>
@@ -4164,8 +4065,8 @@
         <v>100</v>
       </c>
       <c r="BC12" s="30">
-        <f t="array" ref="BC12">_xlfn.RANDARRAY(2,1,12345678,99999999,TRUE)</f>
-        <v>40135841</v>
+        <f t="array" aca="1" ref="BC12" ca="1">_xlfn.RANDARRAY(2,1,12345678,99999999,TRUE)</f>
+        <v>61648916</v>
       </c>
       <c r="BD12" s="17" t="s">
         <v>98</v>
@@ -4207,8 +4108,8 @@
         <v>108</v>
       </c>
       <c r="BQ12" s="13">
-        <f t="array" ref="BQ12">_xlfn.RANDARRAY(2,1,12345,99999,TRUE)</f>
-        <v>12639</v>
+        <f t="array" aca="1" ref="BQ12" ca="1">_xlfn.RANDARRAY(2,1,12345,99999,TRUE)</f>
+        <v>62734</v>
       </c>
       <c r="BR12" s="17">
         <v>44562</v>
@@ -4220,22 +4121,22 @@
         <v>44562</v>
       </c>
       <c r="BU12" s="22">
-        <f t="shared" si="4"/>
-        <v>46168</v>
+        <f t="shared" ca="1" si="4"/>
+        <v>46169</v>
       </c>
       <c r="BV12" s="16" t="s">
         <v>109</v>
       </c>
     </row>
-    <row r="13" ht="15.65" customHeight="1" spans="1:74" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:74" ht="15.65" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="B13" s="10" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="C13" s="11" t="s">
-        <v>161</v>
+        <v>71</v>
       </c>
       <c r="D13" s="12" t="s">
         <v>111</v>
@@ -4244,13 +4145,13 @@
         <v>73</v>
       </c>
       <c r="F13" s="14" t="s">
-        <v>74</v>
+        <v>163</v>
       </c>
       <c r="G13" s="14" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="H13" s="15" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="I13" s="16" t="s">
         <v>77</v>
@@ -4259,8 +4160,8 @@
         <v>78</v>
       </c>
       <c r="K13" s="17">
-        <f t="shared" si="0"/>
-        <v>45796</v>
+        <f t="shared" ca="1" si="0"/>
+        <v>45797</v>
       </c>
       <c r="L13" s="13" t="s">
         <v>73</v>
@@ -4290,8 +4191,8 @@
         <v>78</v>
       </c>
       <c r="U13" s="22">
-        <f t="shared" si="6"/>
-        <v>45703</v>
+        <f t="shared" ca="1" si="6"/>
+        <v>45704</v>
       </c>
       <c r="V13" s="16" t="s">
         <v>83</v>
@@ -4321,7 +4222,7 @@
         <v>89</v>
       </c>
       <c r="AE13" s="33" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="AF13" s="28" t="s">
         <v>89</v>
@@ -4336,26 +4237,26 @@
         <v>89</v>
       </c>
       <c r="AJ13" s="17">
-        <f t="shared" si="7"/>
-        <v>45703</v>
+        <f t="shared" ca="1" si="7"/>
+        <v>45704</v>
       </c>
       <c r="AK13" s="17">
-        <f t="shared" si="7"/>
-        <v>45703</v>
+        <f t="shared" ca="1" si="7"/>
+        <v>45704</v>
       </c>
       <c r="AL13" s="17">
-        <f t="shared" si="7"/>
-        <v>45703</v>
-      </c>
-      <c r="AM13" s="22">
+        <f t="shared" ca="1" si="7"/>
+        <v>45704</v>
+      </c>
+      <c r="AM13" s="22" t="str">
         <f t="shared" si="10"/>
-        <v>NaN</v>
+        <v>N/A</v>
       </c>
       <c r="AN13" s="16" t="s">
         <v>117</v>
       </c>
       <c r="AO13" s="34" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="AP13" s="24" t="s">
         <v>94</v>
@@ -4373,8 +4274,8 @@
         <v>89</v>
       </c>
       <c r="AU13" s="17">
-        <f t="shared" si="3"/>
-        <v>45810</v>
+        <f t="shared" ca="1" si="3"/>
+        <v>45811</v>
       </c>
       <c r="AV13" s="13" t="s">
         <v>73</v>
@@ -4383,8 +4284,8 @@
         <v>97</v>
       </c>
       <c r="AX13" s="30">
-        <f t="array" ref="AX13">_xlfn.RANDARRAY(2,1,1023456789000,9999999999999,TRUE)</f>
-        <v>8813489857973</v>
+        <f t="array" aca="1" ref="AX13" ca="1">_xlfn.RANDARRAY(2,1,1023456789000,9999999999999,TRUE)</f>
+        <v>4366384009376</v>
       </c>
       <c r="AY13" s="17" t="s">
         <v>98</v>
@@ -4399,8 +4300,8 @@
         <v>100</v>
       </c>
       <c r="BC13" s="30">
-        <f t="array" ref="BC13">_xlfn.RANDARRAY(2,1,12345678,99999999,TRUE)</f>
-        <v>87898390</v>
+        <f t="array" aca="1" ref="BC13" ca="1">_xlfn.RANDARRAY(2,1,12345678,99999999,TRUE)</f>
+        <v>27933102</v>
       </c>
       <c r="BD13" s="17" t="s">
         <v>98</v>
@@ -4442,8 +4343,8 @@
         <v>108</v>
       </c>
       <c r="BQ13" s="13">
-        <f t="array" ref="BQ13">_xlfn.RANDARRAY(2,1,12345,99999,TRUE)</f>
-        <v>40203</v>
+        <f t="array" aca="1" ref="BQ13" ca="1">_xlfn.RANDARRAY(2,1,12345,99999,TRUE)</f>
+        <v>78059</v>
       </c>
       <c r="BR13" s="17">
         <v>44562</v>
@@ -4455,19 +4356,23 @@
         <v>44562</v>
       </c>
       <c r="BU13" s="22">
-        <f t="shared" si="4"/>
-        <v>46168</v>
+        <f t="shared" ca="1" si="4"/>
+        <v>46169</v>
       </c>
       <c r="BV13" s="16" t="s">
         <v>109</v>
       </c>
     </row>
-    <row r="14" ht="15.65" customHeight="1" spans="1:74" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:74" ht="15.65" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
-        <v>165</v>
-      </c>
-      <c r="B14" s="10"/>
-      <c r="C14" s="11"/>
+        <v>167</v>
+      </c>
+      <c r="B14" s="10" t="s">
+        <v>168</v>
+      </c>
+      <c r="C14" s="11" t="s">
+        <v>71</v>
+      </c>
       <c r="D14" s="12" t="s">
         <v>111</v>
       </c>
@@ -4475,13 +4380,13 @@
         <v>73</v>
       </c>
       <c r="F14" s="14" t="s">
-        <v>74</v>
+        <v>169</v>
       </c>
       <c r="G14" s="14" t="s">
-        <v>166</v>
+        <v>170</v>
       </c>
       <c r="H14" s="15" t="s">
-        <v>167</v>
+        <v>171</v>
       </c>
       <c r="I14" s="16" t="s">
         <v>77</v>
@@ -4490,8 +4395,8 @@
         <v>78</v>
       </c>
       <c r="K14" s="17">
-        <f t="shared" si="0"/>
-        <v>45796</v>
+        <f t="shared" ca="1" si="0"/>
+        <v>45797</v>
       </c>
       <c r="L14" s="13" t="s">
         <v>73</v>
@@ -4521,8 +4426,8 @@
         <v>78</v>
       </c>
       <c r="U14" s="22">
-        <f t="shared" si="6"/>
-        <v>45703</v>
+        <f t="shared" ca="1" si="6"/>
+        <v>45704</v>
       </c>
       <c r="V14" s="16" t="s">
         <v>83</v>
@@ -4567,26 +4472,26 @@
         <v>89</v>
       </c>
       <c r="AJ14" s="17">
-        <f t="shared" si="7"/>
-        <v>45703</v>
+        <f t="shared" ca="1" si="7"/>
+        <v>45704</v>
       </c>
       <c r="AK14" s="17">
-        <f t="shared" si="7"/>
-        <v>45703</v>
+        <f t="shared" ca="1" si="7"/>
+        <v>45704</v>
       </c>
       <c r="AL14" s="17">
-        <f t="shared" si="7"/>
-        <v>45703</v>
-      </c>
-      <c r="AM14" s="22">
+        <f t="shared" ca="1" si="7"/>
+        <v>45704</v>
+      </c>
+      <c r="AM14" s="22" t="str">
         <f t="shared" ref="AM14:AM17" si="11">AF14</f>
-        <v>NaN</v>
+        <v>N/A</v>
       </c>
       <c r="AN14" s="16" t="s">
         <v>117</v>
       </c>
       <c r="AO14" s="34" t="s">
-        <v>168</v>
+        <v>172</v>
       </c>
       <c r="AP14" s="24" t="s">
         <v>94</v>
@@ -4604,8 +4509,8 @@
         <v>89</v>
       </c>
       <c r="AU14" s="17">
-        <f t="shared" si="3"/>
-        <v>45810</v>
+        <f t="shared" ca="1" si="3"/>
+        <v>45811</v>
       </c>
       <c r="AV14" s="13" t="s">
         <v>73</v>
@@ -4614,8 +4519,8 @@
         <v>97</v>
       </c>
       <c r="AX14" s="30">
-        <f t="array" ref="AX14">_xlfn.RANDARRAY(2,1,1023456789000,9999999999999,TRUE)</f>
-        <v>9815386035281</v>
+        <f t="array" aca="1" ref="AX14" ca="1">_xlfn.RANDARRAY(2,1,1023456789000,9999999999999,TRUE)</f>
+        <v>6437111792437</v>
       </c>
       <c r="AY14" s="17" t="s">
         <v>98</v>
@@ -4630,8 +4535,8 @@
         <v>100</v>
       </c>
       <c r="BC14" s="30">
-        <f t="array" ref="BC14">_xlfn.RANDARRAY(2,1,12345678,99999999,TRUE)</f>
-        <v>29088934</v>
+        <f t="array" aca="1" ref="BC14" ca="1">_xlfn.RANDARRAY(2,1,12345678,99999999,TRUE)</f>
+        <v>77281013</v>
       </c>
       <c r="BD14" s="17" t="s">
         <v>98</v>
@@ -4673,8 +4578,8 @@
         <v>108</v>
       </c>
       <c r="BQ14" s="13">
-        <f t="array" ref="BQ14">_xlfn.RANDARRAY(2,1,12345,99999,TRUE)</f>
-        <v>93717</v>
+        <f t="array" aca="1" ref="BQ14" ca="1">_xlfn.RANDARRAY(2,1,12345,99999,TRUE)</f>
+        <v>49865</v>
       </c>
       <c r="BR14" s="17">
         <v>44562</v>
@@ -4686,19 +4591,23 @@
         <v>44562</v>
       </c>
       <c r="BU14" s="22">
-        <f t="shared" si="4"/>
-        <v>46168</v>
+        <f t="shared" ca="1" si="4"/>
+        <v>46169</v>
       </c>
       <c r="BV14" s="16" t="s">
         <v>109</v>
       </c>
     </row>
-    <row r="15" ht="15.65" customHeight="1" spans="1:74" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:74" ht="15.65" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
-        <v>169</v>
-      </c>
-      <c r="B15" s="10"/>
-      <c r="C15" s="11"/>
+        <v>173</v>
+      </c>
+      <c r="B15" s="10" t="s">
+        <v>174</v>
+      </c>
+      <c r="C15" s="11" t="s">
+        <v>71</v>
+      </c>
       <c r="D15" s="12" t="s">
         <v>111</v>
       </c>
@@ -4706,13 +4615,13 @@
         <v>73</v>
       </c>
       <c r="F15" s="14" t="s">
-        <v>74</v>
+        <v>175</v>
       </c>
       <c r="G15" s="14" t="s">
-        <v>170</v>
+        <v>176</v>
       </c>
       <c r="H15" s="15" t="s">
-        <v>171</v>
+        <v>177</v>
       </c>
       <c r="I15" s="16" t="s">
         <v>77</v>
@@ -4721,8 +4630,8 @@
         <v>78</v>
       </c>
       <c r="K15" s="17">
-        <f t="shared" si="0"/>
-        <v>45796</v>
+        <f t="shared" ca="1" si="0"/>
+        <v>45797</v>
       </c>
       <c r="L15" s="13" t="s">
         <v>73</v>
@@ -4752,8 +4661,8 @@
         <v>78</v>
       </c>
       <c r="U15" s="22">
-        <f t="shared" si="6"/>
-        <v>45703</v>
+        <f t="shared" ca="1" si="6"/>
+        <v>45704</v>
       </c>
       <c r="V15" s="16" t="s">
         <v>83</v>
@@ -4783,7 +4692,7 @@
         <v>89</v>
       </c>
       <c r="AE15" s="33" t="s">
-        <v>172</v>
+        <v>178</v>
       </c>
       <c r="AF15" s="28" t="s">
         <v>89</v>
@@ -4798,26 +4707,26 @@
         <v>89</v>
       </c>
       <c r="AJ15" s="17">
-        <f t="shared" si="7"/>
-        <v>45703</v>
+        <f t="shared" ca="1" si="7"/>
+        <v>45704</v>
       </c>
       <c r="AK15" s="17">
-        <f t="shared" si="7"/>
-        <v>45703</v>
+        <f t="shared" ca="1" si="7"/>
+        <v>45704</v>
       </c>
       <c r="AL15" s="17">
-        <f t="shared" si="7"/>
-        <v>45703</v>
-      </c>
-      <c r="AM15" s="22">
+        <f t="shared" ca="1" si="7"/>
+        <v>45704</v>
+      </c>
+      <c r="AM15" s="22" t="str">
         <f t="shared" si="11"/>
-        <v>NaN</v>
+        <v>N/A</v>
       </c>
       <c r="AN15" s="16" t="s">
         <v>117</v>
       </c>
       <c r="AO15" s="34" t="s">
-        <v>173</v>
+        <v>179</v>
       </c>
       <c r="AP15" s="24" t="s">
         <v>94</v>
@@ -4835,8 +4744,8 @@
         <v>89</v>
       </c>
       <c r="AU15" s="17">
-        <f t="shared" si="3"/>
-        <v>45810</v>
+        <f t="shared" ca="1" si="3"/>
+        <v>45811</v>
       </c>
       <c r="AV15" s="13" t="s">
         <v>73</v>
@@ -4845,8 +4754,8 @@
         <v>97</v>
       </c>
       <c r="AX15" s="30">
-        <f t="array" ref="AX15">_xlfn.RANDARRAY(2,1,1023456789000,9999999999999,TRUE)</f>
-        <v>1873131984301</v>
+        <f t="array" aca="1" ref="AX15" ca="1">_xlfn.RANDARRAY(2,1,1023456789000,9999999999999,TRUE)</f>
+        <v>8792712949859</v>
       </c>
       <c r="AY15" s="17" t="s">
         <v>98</v>
@@ -4861,8 +4770,8 @@
         <v>100</v>
       </c>
       <c r="BC15" s="30">
-        <f t="array" ref="BC15">_xlfn.RANDARRAY(2,1,12345678,99999999,TRUE)</f>
-        <v>12695563</v>
+        <f t="array" aca="1" ref="BC15" ca="1">_xlfn.RANDARRAY(2,1,12345678,99999999,TRUE)</f>
+        <v>17984405</v>
       </c>
       <c r="BD15" s="17" t="s">
         <v>98</v>
@@ -4904,8 +4813,8 @@
         <v>108</v>
       </c>
       <c r="BQ15" s="13">
-        <f t="array" ref="BQ15">_xlfn.RANDARRAY(2,1,12345,99999,TRUE)</f>
-        <v>55204</v>
+        <f t="array" aca="1" ref="BQ15" ca="1">_xlfn.RANDARRAY(2,1,12345,99999,TRUE)</f>
+        <v>27486</v>
       </c>
       <c r="BR15" s="17">
         <v>44562</v>
@@ -4917,19 +4826,23 @@
         <v>44562</v>
       </c>
       <c r="BU15" s="22">
-        <f t="shared" si="4"/>
-        <v>46168</v>
+        <f t="shared" ca="1" si="4"/>
+        <v>46169</v>
       </c>
       <c r="BV15" s="16" t="s">
         <v>109</v>
       </c>
     </row>
-    <row r="16" ht="15.65" customHeight="1" spans="1:74" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:74" ht="15.65" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
-        <v>174</v>
-      </c>
-      <c r="B16" s="10"/>
-      <c r="C16" s="11"/>
+        <v>180</v>
+      </c>
+      <c r="B16" s="10" t="s">
+        <v>181</v>
+      </c>
+      <c r="C16" s="11" t="s">
+        <v>71</v>
+      </c>
       <c r="D16" s="12" t="s">
         <v>111</v>
       </c>
@@ -4937,13 +4850,13 @@
         <v>73</v>
       </c>
       <c r="F16" s="14" t="s">
-        <v>74</v>
+        <v>182</v>
       </c>
       <c r="G16" s="14" t="s">
-        <v>175</v>
+        <v>183</v>
       </c>
       <c r="H16" s="15" t="s">
-        <v>176</v>
+        <v>184</v>
       </c>
       <c r="I16" s="16" t="s">
         <v>77</v>
@@ -4952,8 +4865,8 @@
         <v>78</v>
       </c>
       <c r="K16" s="17">
-        <f t="shared" si="0"/>
-        <v>45796</v>
+        <f t="shared" ca="1" si="0"/>
+        <v>45797</v>
       </c>
       <c r="L16" s="13" t="s">
         <v>73</v>
@@ -4983,8 +4896,8 @@
         <v>78</v>
       </c>
       <c r="U16" s="22">
-        <f t="shared" si="6"/>
-        <v>45703</v>
+        <f t="shared" ca="1" si="6"/>
+        <v>45704</v>
       </c>
       <c r="V16" s="16" t="s">
         <v>83</v>
@@ -5029,26 +4942,26 @@
         <v>89</v>
       </c>
       <c r="AJ16" s="17">
-        <f t="shared" si="7"/>
-        <v>45703</v>
+        <f t="shared" ca="1" si="7"/>
+        <v>45704</v>
       </c>
       <c r="AK16" s="17">
-        <f t="shared" si="7"/>
-        <v>45703</v>
+        <f t="shared" ca="1" si="7"/>
+        <v>45704</v>
       </c>
       <c r="AL16" s="17">
-        <f t="shared" si="7"/>
-        <v>45703</v>
-      </c>
-      <c r="AM16" s="22">
+        <f t="shared" ca="1" si="7"/>
+        <v>45704</v>
+      </c>
+      <c r="AM16" s="22" t="str">
         <f t="shared" si="11"/>
-        <v>NaN</v>
+        <v>N/A</v>
       </c>
       <c r="AN16" s="16" t="s">
         <v>117</v>
       </c>
       <c r="AO16" s="34" t="s">
-        <v>177</v>
+        <v>185</v>
       </c>
       <c r="AP16" s="24" t="s">
         <v>94</v>
@@ -5066,8 +4979,8 @@
         <v>89</v>
       </c>
       <c r="AU16" s="17">
-        <f t="shared" si="3"/>
-        <v>45810</v>
+        <f t="shared" ca="1" si="3"/>
+        <v>45811</v>
       </c>
       <c r="AV16" s="13" t="s">
         <v>73</v>
@@ -5076,8 +4989,8 @@
         <v>97</v>
       </c>
       <c r="AX16" s="30">
-        <f t="array" ref="AX16">_xlfn.RANDARRAY(2,1,1023456789000,9999999999999,TRUE)</f>
-        <v>7672881210087</v>
+        <f t="array" aca="1" ref="AX16" ca="1">_xlfn.RANDARRAY(2,1,1023456789000,9999999999999,TRUE)</f>
+        <v>5504649388526</v>
       </c>
       <c r="AY16" s="17" t="s">
         <v>98</v>
@@ -5092,8 +5005,8 @@
         <v>100</v>
       </c>
       <c r="BC16" s="30">
-        <f t="array" ref="BC16">_xlfn.RANDARRAY(2,1,12345678,99999999,TRUE)</f>
-        <v>30907114</v>
+        <f t="array" aca="1" ref="BC16" ca="1">_xlfn.RANDARRAY(2,1,12345678,99999999,TRUE)</f>
+        <v>68346885</v>
       </c>
       <c r="BD16" s="17" t="s">
         <v>98</v>
@@ -5135,8 +5048,8 @@
         <v>108</v>
       </c>
       <c r="BQ16" s="13">
-        <f t="array" ref="BQ16">_xlfn.RANDARRAY(2,1,12345,99999,TRUE)</f>
-        <v>31270</v>
+        <f t="array" aca="1" ref="BQ16" ca="1">_xlfn.RANDARRAY(2,1,12345,99999,TRUE)</f>
+        <v>57148</v>
       </c>
       <c r="BR16" s="17">
         <v>44562</v>
@@ -5148,19 +5061,23 @@
         <v>44562</v>
       </c>
       <c r="BU16" s="22">
-        <f t="shared" si="4"/>
-        <v>46168</v>
+        <f t="shared" ca="1" si="4"/>
+        <v>46169</v>
       </c>
       <c r="BV16" s="16" t="s">
         <v>109</v>
       </c>
     </row>
-    <row r="17" ht="15.65" customHeight="1" spans="1:74" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:74" ht="15.65" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
-        <v>178</v>
-      </c>
-      <c r="B17" s="10"/>
-      <c r="C17" s="11"/>
+        <v>186</v>
+      </c>
+      <c r="B17" s="10" t="s">
+        <v>187</v>
+      </c>
+      <c r="C17" s="11" t="s">
+        <v>71</v>
+      </c>
       <c r="D17" s="12" t="s">
         <v>111</v>
       </c>
@@ -5168,13 +5085,13 @@
         <v>73</v>
       </c>
       <c r="F17" s="14" t="s">
-        <v>74</v>
+        <v>188</v>
       </c>
       <c r="G17" s="14" t="s">
-        <v>179</v>
+        <v>189</v>
       </c>
       <c r="H17" s="15" t="s">
-        <v>180</v>
+        <v>190</v>
       </c>
       <c r="I17" s="16" t="s">
         <v>77</v>
@@ -5183,8 +5100,8 @@
         <v>78</v>
       </c>
       <c r="K17" s="17">
-        <f t="shared" si="0"/>
-        <v>45796</v>
+        <f t="shared" ca="1" si="0"/>
+        <v>45797</v>
       </c>
       <c r="L17" s="13" t="s">
         <v>73</v>
@@ -5214,8 +5131,8 @@
         <v>78</v>
       </c>
       <c r="U17" s="22">
-        <f t="shared" si="6"/>
-        <v>45703</v>
+        <f t="shared" ca="1" si="6"/>
+        <v>45704</v>
       </c>
       <c r="V17" s="16" t="s">
         <v>83</v>
@@ -5260,26 +5177,26 @@
         <v>89</v>
       </c>
       <c r="AJ17" s="17">
-        <f t="shared" si="7"/>
-        <v>45703</v>
+        <f t="shared" ca="1" si="7"/>
+        <v>45704</v>
       </c>
       <c r="AK17" s="17">
-        <f t="shared" si="7"/>
-        <v>45703</v>
+        <f t="shared" ca="1" si="7"/>
+        <v>45704</v>
       </c>
       <c r="AL17" s="17">
-        <f t="shared" si="7"/>
-        <v>45703</v>
-      </c>
-      <c r="AM17" s="22">
+        <f t="shared" ca="1" si="7"/>
+        <v>45704</v>
+      </c>
+      <c r="AM17" s="22" t="str">
         <f t="shared" si="11"/>
-        <v>NaN</v>
+        <v>N/A</v>
       </c>
       <c r="AN17" s="16" t="s">
         <v>117</v>
       </c>
       <c r="AO17" s="34" t="s">
-        <v>181</v>
+        <v>191</v>
       </c>
       <c r="AP17" s="24" t="s">
         <v>94</v>
@@ -5297,8 +5214,8 @@
         <v>89</v>
       </c>
       <c r="AU17" s="17">
-        <f t="shared" si="3"/>
-        <v>45810</v>
+        <f t="shared" ca="1" si="3"/>
+        <v>45811</v>
       </c>
       <c r="AV17" s="13" t="s">
         <v>73</v>
@@ -5307,8 +5224,8 @@
         <v>97</v>
       </c>
       <c r="AX17" s="30">
-        <f t="array" ref="AX17">_xlfn.RANDARRAY(2,1,1023456789000,9999999999999,TRUE)</f>
-        <v>2852836738206</v>
+        <f t="array" aca="1" ref="AX17" ca="1">_xlfn.RANDARRAY(2,1,1023456789000,9999999999999,TRUE)</f>
+        <v>3757536959112</v>
       </c>
       <c r="AY17" s="17" t="s">
         <v>98</v>
@@ -5323,8 +5240,8 @@
         <v>100</v>
       </c>
       <c r="BC17" s="30">
-        <f t="array" ref="BC17">_xlfn.RANDARRAY(2,1,12345678,99999999,TRUE)</f>
-        <v>91987166</v>
+        <f t="array" aca="1" ref="BC17" ca="1">_xlfn.RANDARRAY(2,1,12345678,99999999,TRUE)</f>
+        <v>47464747</v>
       </c>
       <c r="BD17" s="17" t="s">
         <v>98</v>
@@ -5366,8 +5283,8 @@
         <v>108</v>
       </c>
       <c r="BQ17" s="13">
-        <f t="array" ref="BQ17">_xlfn.RANDARRAY(2,1,12345,99999,TRUE)</f>
-        <v>50534</v>
+        <f t="array" aca="1" ref="BQ17" ca="1">_xlfn.RANDARRAY(2,1,12345,99999,TRUE)</f>
+        <v>79607</v>
       </c>
       <c r="BR17" s="17">
         <v>44562</v>
@@ -5379,19 +5296,23 @@
         <v>44562</v>
       </c>
       <c r="BU17" s="22">
-        <f t="shared" si="4"/>
-        <v>46168</v>
+        <f t="shared" ca="1" si="4"/>
+        <v>46169</v>
       </c>
       <c r="BV17" s="16" t="s">
         <v>109</v>
       </c>
     </row>
-    <row r="18" ht="15.65" customHeight="1" spans="1:74" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:74" ht="15.65" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
-        <v>182</v>
-      </c>
-      <c r="B18" s="10"/>
-      <c r="C18" s="11"/>
+        <v>192</v>
+      </c>
+      <c r="B18" s="10">
+        <v>10699364</v>
+      </c>
+      <c r="C18" s="11" t="s">
+        <v>71</v>
+      </c>
       <c r="D18" s="12" t="s">
         <v>111</v>
       </c>
@@ -5399,13 +5320,13 @@
         <v>73</v>
       </c>
       <c r="F18" s="14" t="s">
-        <v>74</v>
+        <v>193</v>
       </c>
       <c r="G18" s="14" t="s">
-        <v>183</v>
+        <v>194</v>
       </c>
       <c r="H18" s="15" t="s">
-        <v>184</v>
+        <v>195</v>
       </c>
       <c r="I18" s="16" t="s">
         <v>77</v>
@@ -5414,8 +5335,8 @@
         <v>78</v>
       </c>
       <c r="K18" s="17">
-        <f t="shared" si="0"/>
-        <v>45796</v>
+        <f t="shared" ca="1" si="0"/>
+        <v>45797</v>
       </c>
       <c r="L18" s="13" t="s">
         <v>73</v>
@@ -5445,8 +5366,8 @@
         <v>78</v>
       </c>
       <c r="U18" s="22">
-        <f t="shared" si="6"/>
-        <v>45703</v>
+        <f t="shared" ca="1" si="6"/>
+        <v>45704</v>
       </c>
       <c r="V18" s="16" t="s">
         <v>83</v>
@@ -5491,26 +5412,26 @@
         <v>89</v>
       </c>
       <c r="AJ18" s="17">
-        <f t="shared" si="7"/>
-        <v>45703</v>
+        <f t="shared" ca="1" si="7"/>
+        <v>45704</v>
       </c>
       <c r="AK18" s="17">
-        <f t="shared" si="7"/>
-        <v>45703</v>
+        <f t="shared" ca="1" si="7"/>
+        <v>45704</v>
       </c>
       <c r="AL18" s="17">
-        <f t="shared" si="7"/>
-        <v>45703</v>
-      </c>
-      <c r="AM18" s="22">
+        <f t="shared" ca="1" si="7"/>
+        <v>45704</v>
+      </c>
+      <c r="AM18" s="22" t="str">
         <f t="shared" ref="AM18:AM21" si="12">AF18</f>
-        <v>NaN</v>
+        <v>N/A</v>
       </c>
       <c r="AN18" s="16" t="s">
         <v>117</v>
       </c>
       <c r="AO18" s="34" t="s">
-        <v>185</v>
+        <v>196</v>
       </c>
       <c r="AP18" s="24" t="s">
         <v>94</v>
@@ -5528,8 +5449,8 @@
         <v>89</v>
       </c>
       <c r="AU18" s="17">
-        <f t="shared" si="3"/>
-        <v>45810</v>
+        <f t="shared" ca="1" si="3"/>
+        <v>45811</v>
       </c>
       <c r="AV18" s="13" t="s">
         <v>73</v>
@@ -5538,8 +5459,8 @@
         <v>97</v>
       </c>
       <c r="AX18" s="30">
-        <f t="array" ref="AX18">_xlfn.RANDARRAY(2,1,1023456789000,9999999999999,TRUE)</f>
-        <v>9499744009766</v>
+        <f t="array" aca="1" ref="AX18" ca="1">_xlfn.RANDARRAY(2,1,1023456789000,9999999999999,TRUE)</f>
+        <v>5799185247674</v>
       </c>
       <c r="AY18" s="17" t="s">
         <v>98</v>
@@ -5554,8 +5475,8 @@
         <v>100</v>
       </c>
       <c r="BC18" s="30">
-        <f t="array" ref="BC18">_xlfn.RANDARRAY(2,1,12345678,99999999,TRUE)</f>
-        <v>94678553</v>
+        <f t="array" aca="1" ref="BC18" ca="1">_xlfn.RANDARRAY(2,1,12345678,99999999,TRUE)</f>
+        <v>85064072</v>
       </c>
       <c r="BD18" s="17" t="s">
         <v>98</v>
@@ -5597,8 +5518,8 @@
         <v>108</v>
       </c>
       <c r="BQ18" s="13">
-        <f t="array" ref="BQ18">_xlfn.RANDARRAY(2,1,12345,99999,TRUE)</f>
-        <v>32829</v>
+        <f t="array" aca="1" ref="BQ18" ca="1">_xlfn.RANDARRAY(2,1,12345,99999,TRUE)</f>
+        <v>41158</v>
       </c>
       <c r="BR18" s="17">
         <v>44562</v>
@@ -5610,19 +5531,23 @@
         <v>44562</v>
       </c>
       <c r="BU18" s="22">
-        <f t="shared" si="4"/>
-        <v>46168</v>
+        <f t="shared" ca="1" si="4"/>
+        <v>46169</v>
       </c>
       <c r="BV18" s="16" t="s">
         <v>109</v>
       </c>
     </row>
-    <row r="19" ht="15.65" customHeight="1" spans="1:74" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:74" ht="15.65" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
-        <v>186</v>
-      </c>
-      <c r="B19" s="10"/>
-      <c r="C19" s="11"/>
+        <v>197</v>
+      </c>
+      <c r="B19" s="10" t="s">
+        <v>198</v>
+      </c>
+      <c r="C19" s="11" t="s">
+        <v>71</v>
+      </c>
       <c r="D19" s="12" t="s">
         <v>111</v>
       </c>
@@ -5630,13 +5555,13 @@
         <v>73</v>
       </c>
       <c r="F19" s="14" t="s">
-        <v>74</v>
+        <v>199</v>
       </c>
       <c r="G19" s="14" t="s">
-        <v>187</v>
+        <v>200</v>
       </c>
       <c r="H19" s="15" t="s">
-        <v>188</v>
+        <v>201</v>
       </c>
       <c r="I19" s="16" t="s">
         <v>77</v>
@@ -5645,8 +5570,8 @@
         <v>78</v>
       </c>
       <c r="K19" s="17">
-        <f t="shared" si="0"/>
-        <v>45796</v>
+        <f t="shared" ca="1" si="0"/>
+        <v>45797</v>
       </c>
       <c r="L19" s="13" t="s">
         <v>73</v>
@@ -5676,8 +5601,8 @@
         <v>78</v>
       </c>
       <c r="U19" s="22">
-        <f t="shared" si="6"/>
-        <v>45703</v>
+        <f t="shared" ca="1" si="6"/>
+        <v>45704</v>
       </c>
       <c r="V19" s="16" t="s">
         <v>83</v>
@@ -5722,26 +5647,26 @@
         <v>89</v>
       </c>
       <c r="AJ19" s="17">
-        <f t="shared" si="7"/>
-        <v>45703</v>
+        <f t="shared" ca="1" si="7"/>
+        <v>45704</v>
       </c>
       <c r="AK19" s="17">
-        <f t="shared" si="7"/>
-        <v>45703</v>
+        <f t="shared" ca="1" si="7"/>
+        <v>45704</v>
       </c>
       <c r="AL19" s="17">
-        <f t="shared" si="7"/>
-        <v>45703</v>
-      </c>
-      <c r="AM19" s="22">
+        <f t="shared" ca="1" si="7"/>
+        <v>45704</v>
+      </c>
+      <c r="AM19" s="22" t="str">
         <f t="shared" si="12"/>
-        <v>NaN</v>
+        <v>N/A</v>
       </c>
       <c r="AN19" s="16" t="s">
         <v>117</v>
       </c>
       <c r="AO19" s="34" t="s">
-        <v>189</v>
+        <v>202</v>
       </c>
       <c r="AP19" s="24" t="s">
         <v>94</v>
@@ -5759,8 +5684,8 @@
         <v>89</v>
       </c>
       <c r="AU19" s="17">
-        <f t="shared" si="3"/>
-        <v>45810</v>
+        <f t="shared" ca="1" si="3"/>
+        <v>45811</v>
       </c>
       <c r="AV19" s="13" t="s">
         <v>73</v>
@@ -5769,8 +5694,8 @@
         <v>97</v>
       </c>
       <c r="AX19" s="30">
-        <f t="array" ref="AX19">_xlfn.RANDARRAY(2,1,1023456789000,9999999999999,TRUE)</f>
-        <v>9962487128994</v>
+        <f t="array" aca="1" ref="AX19" ca="1">_xlfn.RANDARRAY(2,1,1023456789000,9999999999999,TRUE)</f>
+        <v>1237615080180</v>
       </c>
       <c r="AY19" s="17" t="s">
         <v>98</v>
@@ -5785,8 +5710,8 @@
         <v>100</v>
       </c>
       <c r="BC19" s="30">
-        <f t="array" ref="BC19">_xlfn.RANDARRAY(2,1,12345678,99999999,TRUE)</f>
-        <v>71195776</v>
+        <f t="array" aca="1" ref="BC19" ca="1">_xlfn.RANDARRAY(2,1,12345678,99999999,TRUE)</f>
+        <v>20700790</v>
       </c>
       <c r="BD19" s="17" t="s">
         <v>98</v>
@@ -5828,8 +5753,8 @@
         <v>108</v>
       </c>
       <c r="BQ19" s="13">
-        <f t="array" ref="BQ19">_xlfn.RANDARRAY(2,1,12345,99999,TRUE)</f>
-        <v>41850</v>
+        <f t="array" aca="1" ref="BQ19" ca="1">_xlfn.RANDARRAY(2,1,12345,99999,TRUE)</f>
+        <v>48660</v>
       </c>
       <c r="BR19" s="17">
         <v>44562</v>
@@ -5841,19 +5766,23 @@
         <v>44562</v>
       </c>
       <c r="BU19" s="22">
-        <f t="shared" si="4"/>
-        <v>46168</v>
+        <f t="shared" ca="1" si="4"/>
+        <v>46169</v>
       </c>
       <c r="BV19" s="16" t="s">
         <v>109</v>
       </c>
     </row>
-    <row r="20" ht="15.65" customHeight="1" spans="1:74" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:74" ht="15.65" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
-        <v>190</v>
-      </c>
-      <c r="B20" s="10"/>
-      <c r="C20" s="11"/>
+        <v>203</v>
+      </c>
+      <c r="B20" s="10" t="s">
+        <v>204</v>
+      </c>
+      <c r="C20" s="11" t="s">
+        <v>71</v>
+      </c>
       <c r="D20" s="12" t="s">
         <v>111</v>
       </c>
@@ -5861,13 +5790,13 @@
         <v>73</v>
       </c>
       <c r="F20" s="14" t="s">
-        <v>74</v>
+        <v>205</v>
       </c>
       <c r="G20" s="14" t="s">
-        <v>191</v>
+        <v>206</v>
       </c>
       <c r="H20" s="15" t="s">
-        <v>192</v>
+        <v>207</v>
       </c>
       <c r="I20" s="16" t="s">
         <v>77</v>
@@ -5876,8 +5805,8 @@
         <v>78</v>
       </c>
       <c r="K20" s="17">
-        <f t="shared" si="0"/>
-        <v>45796</v>
+        <f t="shared" ca="1" si="0"/>
+        <v>45797</v>
       </c>
       <c r="L20" s="13" t="s">
         <v>73</v>
@@ -5907,8 +5836,8 @@
         <v>78</v>
       </c>
       <c r="U20" s="22">
-        <f t="shared" si="6"/>
-        <v>45703</v>
+        <f t="shared" ca="1" si="6"/>
+        <v>45704</v>
       </c>
       <c r="V20" s="16" t="s">
         <v>83</v>
@@ -5938,7 +5867,7 @@
         <v>89</v>
       </c>
       <c r="AE20" s="33" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="AF20" s="28" t="s">
         <v>89</v>
@@ -5953,26 +5882,26 @@
         <v>89</v>
       </c>
       <c r="AJ20" s="17">
-        <f t="shared" si="7"/>
-        <v>45703</v>
+        <f t="shared" ca="1" si="7"/>
+        <v>45704</v>
       </c>
       <c r="AK20" s="17">
-        <f t="shared" si="7"/>
-        <v>45703</v>
+        <f t="shared" ca="1" si="7"/>
+        <v>45704</v>
       </c>
       <c r="AL20" s="17">
-        <f t="shared" si="7"/>
-        <v>45703</v>
-      </c>
-      <c r="AM20" s="22">
+        <f t="shared" ca="1" si="7"/>
+        <v>45704</v>
+      </c>
+      <c r="AM20" s="22" t="str">
         <f t="shared" si="12"/>
-        <v>NaN</v>
+        <v>N/A</v>
       </c>
       <c r="AN20" s="16" t="s">
         <v>117</v>
       </c>
       <c r="AO20" s="34" t="s">
-        <v>193</v>
+        <v>208</v>
       </c>
       <c r="AP20" s="24" t="s">
         <v>94</v>
@@ -5990,8 +5919,8 @@
         <v>89</v>
       </c>
       <c r="AU20" s="17">
-        <f t="shared" si="3"/>
-        <v>45810</v>
+        <f t="shared" ca="1" si="3"/>
+        <v>45811</v>
       </c>
       <c r="AV20" s="13" t="s">
         <v>73</v>
@@ -6000,8 +5929,8 @@
         <v>97</v>
       </c>
       <c r="AX20" s="30">
-        <f t="array" ref="AX20">_xlfn.RANDARRAY(2,1,1023456789000,9999999999999,TRUE)</f>
-        <v>5536392931674</v>
+        <f t="array" aca="1" ref="AX20" ca="1">_xlfn.RANDARRAY(2,1,1023456789000,9999999999999,TRUE)</f>
+        <v>9357638217148</v>
       </c>
       <c r="AY20" s="17" t="s">
         <v>98</v>
@@ -6016,8 +5945,8 @@
         <v>100</v>
       </c>
       <c r="BC20" s="30">
-        <f t="array" ref="BC20">_xlfn.RANDARRAY(2,1,12345678,99999999,TRUE)</f>
-        <v>86167326</v>
+        <f t="array" aca="1" ref="BC20" ca="1">_xlfn.RANDARRAY(2,1,12345678,99999999,TRUE)</f>
+        <v>46232408</v>
       </c>
       <c r="BD20" s="17" t="s">
         <v>98</v>
@@ -6059,8 +5988,8 @@
         <v>108</v>
       </c>
       <c r="BQ20" s="13">
-        <f t="array" ref="BQ20">_xlfn.RANDARRAY(2,1,12345,99999,TRUE)</f>
-        <v>92985</v>
+        <f t="array" aca="1" ref="BQ20" ca="1">_xlfn.RANDARRAY(2,1,12345,99999,TRUE)</f>
+        <v>93830</v>
       </c>
       <c r="BR20" s="17">
         <v>44562</v>
@@ -6072,19 +6001,23 @@
         <v>44562</v>
       </c>
       <c r="BU20" s="22">
-        <f t="shared" si="4"/>
-        <v>46168</v>
+        <f t="shared" ca="1" si="4"/>
+        <v>46169</v>
       </c>
       <c r="BV20" s="16" t="s">
         <v>109</v>
       </c>
     </row>
-    <row r="21" ht="15.65" customHeight="1" spans="1:74" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:74" ht="15.65" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
-        <v>194</v>
-      </c>
-      <c r="B21" s="10"/>
-      <c r="C21" s="11"/>
+        <v>209</v>
+      </c>
+      <c r="B21" s="10" t="s">
+        <v>210</v>
+      </c>
+      <c r="C21" s="11" t="s">
+        <v>71</v>
+      </c>
       <c r="D21" s="12" t="s">
         <v>111</v>
       </c>
@@ -6092,13 +6025,13 @@
         <v>73</v>
       </c>
       <c r="F21" s="14" t="s">
-        <v>74</v>
+        <v>211</v>
       </c>
       <c r="G21" s="14" t="s">
-        <v>195</v>
+        <v>212</v>
       </c>
       <c r="H21" s="15" t="s">
-        <v>196</v>
+        <v>213</v>
       </c>
       <c r="I21" s="16" t="s">
         <v>77</v>
@@ -6107,8 +6040,8 @@
         <v>78</v>
       </c>
       <c r="K21" s="17">
-        <f t="shared" si="0"/>
-        <v>45796</v>
+        <f t="shared" ca="1" si="0"/>
+        <v>45797</v>
       </c>
       <c r="L21" s="13" t="s">
         <v>73</v>
@@ -6138,8 +6071,8 @@
         <v>78</v>
       </c>
       <c r="U21" s="22">
-        <f t="shared" si="6"/>
-        <v>45703</v>
+        <f t="shared" ca="1" si="6"/>
+        <v>45704</v>
       </c>
       <c r="V21" s="16" t="s">
         <v>83</v>
@@ -6169,7 +6102,7 @@
         <v>89</v>
       </c>
       <c r="AE21" s="33" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="AF21" s="28" t="s">
         <v>89</v>
@@ -6184,26 +6117,26 @@
         <v>89</v>
       </c>
       <c r="AJ21" s="17">
-        <f t="shared" si="7"/>
-        <v>45703</v>
+        <f t="shared" ca="1" si="7"/>
+        <v>45704</v>
       </c>
       <c r="AK21" s="17">
-        <f t="shared" si="7"/>
-        <v>45703</v>
+        <f t="shared" ca="1" si="7"/>
+        <v>45704</v>
       </c>
       <c r="AL21" s="17">
-        <f t="shared" si="7"/>
-        <v>45703</v>
-      </c>
-      <c r="AM21" s="22">
+        <f t="shared" ca="1" si="7"/>
+        <v>45704</v>
+      </c>
+      <c r="AM21" s="22" t="str">
         <f t="shared" si="12"/>
-        <v>NaN</v>
+        <v>N/A</v>
       </c>
       <c r="AN21" s="16" t="s">
         <v>117</v>
       </c>
       <c r="AO21" s="34" t="s">
-        <v>168</v>
+        <v>172</v>
       </c>
       <c r="AP21" s="24" t="s">
         <v>94</v>
@@ -6221,8 +6154,8 @@
         <v>89</v>
       </c>
       <c r="AU21" s="17">
-        <f t="shared" si="3"/>
-        <v>45810</v>
+        <f t="shared" ca="1" si="3"/>
+        <v>45811</v>
       </c>
       <c r="AV21" s="13" t="s">
         <v>73</v>
@@ -6231,8 +6164,8 @@
         <v>97</v>
       </c>
       <c r="AX21" s="30">
-        <f t="array" ref="AX21">_xlfn.RANDARRAY(2,1,1023456789000,9999999999999,TRUE)</f>
-        <v>4090724590299</v>
+        <f t="array" aca="1" ref="AX21" ca="1">_xlfn.RANDARRAY(2,1,1023456789000,9999999999999,TRUE)</f>
+        <v>8944115535401</v>
       </c>
       <c r="AY21" s="17" t="s">
         <v>98</v>
@@ -6247,8 +6180,8 @@
         <v>100</v>
       </c>
       <c r="BC21" s="30">
-        <f t="array" ref="BC21">_xlfn.RANDARRAY(2,1,12345678,99999999,TRUE)</f>
-        <v>19527257</v>
+        <f t="array" aca="1" ref="BC21" ca="1">_xlfn.RANDARRAY(2,1,12345678,99999999,TRUE)</f>
+        <v>99244537</v>
       </c>
       <c r="BD21" s="17" t="s">
         <v>98</v>
@@ -6290,8 +6223,8 @@
         <v>108</v>
       </c>
       <c r="BQ21" s="13">
-        <f t="array" ref="BQ21">_xlfn.RANDARRAY(2,1,12345,99999,TRUE)</f>
-        <v>45483</v>
+        <f t="array" aca="1" ref="BQ21" ca="1">_xlfn.RANDARRAY(2,1,12345,99999,TRUE)</f>
+        <v>51113</v>
       </c>
       <c r="BR21" s="17">
         <v>44562</v>
@@ -6303,76 +6236,47 @@
         <v>44562</v>
       </c>
       <c r="BU21" s="22">
-        <f t="shared" si="4"/>
-        <v>46168</v>
+        <f t="shared" ca="1" si="4"/>
+        <v>46169</v>
       </c>
       <c r="BV21" s="16" t="s">
         <v>109</v>
       </c>
     </row>
   </sheetData>
-  <dataValidations count="12">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AH10:AH21">
+  <autoFilter ref="A1:BV21" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
+  <dataValidations count="2">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AH10:AH21 V10:V21 T10:T21 Q10:Q21 J10:J21 BL10:BL21" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>INDIRECT($E2)</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AH2:AH21">
-      <formula1>INDIRECT($E2)</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BL10:BL21">
-      <formula1>INDIRECT($E2)</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="BL2:BL21">
-      <formula1>INDIRECT($E2)</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J10:J21">
-      <formula1>INDIRECT($E2)</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J2:J21">
-      <formula1>INDIRECT($E2)</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="Q10:Q21">
-      <formula1>INDIRECT($E2)</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="Q2:Q21">
-      <formula1>INDIRECT($E2)</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="T10:T21">
-      <formula1>INDIRECT($E2)</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="T2:T21">
-      <formula1>INDIRECT($E2)</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="V10:V21">
-      <formula1>INDIRECT($E2)</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="V2:V21">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AH2:AH21 V2:V21 T2:T21 Q2:Q21 J2:J21 BL2:BL21" xr:uid="{00000000-0002-0000-0000-000001000000}">
       <formula1>INDIRECT($E2)</formula1>
     </dataValidation>
   </dataValidations>
   <hyperlinks>
-    <hyperlink ref="S2" r:id="rId1"/>
-    <hyperlink ref="S3" r:id="rId2"/>
-    <hyperlink ref="S4" r:id="rId3"/>
-    <hyperlink ref="S5" r:id="rId4"/>
-    <hyperlink ref="S6" r:id="rId5"/>
-    <hyperlink ref="S7" r:id="rId6"/>
-    <hyperlink ref="S8" r:id="rId7"/>
-    <hyperlink ref="S9" r:id="rId8"/>
-    <hyperlink ref="S10" r:id="rId9"/>
-    <hyperlink ref="S11" r:id="rId10"/>
-    <hyperlink ref="S12" r:id="rId11"/>
-    <hyperlink ref="S13" r:id="rId12"/>
-    <hyperlink ref="S14" r:id="rId13"/>
-    <hyperlink ref="S15" r:id="rId14"/>
-    <hyperlink ref="S16" r:id="rId15"/>
-    <hyperlink ref="S17" r:id="rId16"/>
-    <hyperlink ref="S18" r:id="rId17"/>
-    <hyperlink ref="S19" r:id="rId18"/>
-    <hyperlink ref="S20" r:id="rId19"/>
-    <hyperlink ref="S21" r:id="rId20"/>
+    <hyperlink ref="S2" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
+    <hyperlink ref="S3" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
+    <hyperlink ref="S4" r:id="rId3" xr:uid="{00000000-0004-0000-0000-000002000000}"/>
+    <hyperlink ref="S5" r:id="rId4" xr:uid="{00000000-0004-0000-0000-000003000000}"/>
+    <hyperlink ref="S6" r:id="rId5" xr:uid="{00000000-0004-0000-0000-000004000000}"/>
+    <hyperlink ref="S7" r:id="rId6" xr:uid="{00000000-0004-0000-0000-000005000000}"/>
+    <hyperlink ref="S8" r:id="rId7" xr:uid="{00000000-0004-0000-0000-000006000000}"/>
+    <hyperlink ref="S9" r:id="rId8" xr:uid="{00000000-0004-0000-0000-000007000000}"/>
+    <hyperlink ref="S10" r:id="rId9" xr:uid="{00000000-0004-0000-0000-000008000000}"/>
+    <hyperlink ref="S11" r:id="rId10" xr:uid="{00000000-0004-0000-0000-000009000000}"/>
+    <hyperlink ref="S12" r:id="rId11" xr:uid="{00000000-0004-0000-0000-00000A000000}"/>
+    <hyperlink ref="S13" r:id="rId12" xr:uid="{00000000-0004-0000-0000-00000B000000}"/>
+    <hyperlink ref="S14" r:id="rId13" xr:uid="{00000000-0004-0000-0000-00000C000000}"/>
+    <hyperlink ref="S15" r:id="rId14" xr:uid="{00000000-0004-0000-0000-00000D000000}"/>
+    <hyperlink ref="S16" r:id="rId15" xr:uid="{00000000-0004-0000-0000-00000E000000}"/>
+    <hyperlink ref="S17" r:id="rId16" xr:uid="{00000000-0004-0000-0000-00000F000000}"/>
+    <hyperlink ref="S18" r:id="rId17" xr:uid="{00000000-0004-0000-0000-000010000000}"/>
+    <hyperlink ref="S19" r:id="rId18" xr:uid="{00000000-0004-0000-0000-000011000000}"/>
+    <hyperlink ref="S20" r:id="rId19" xr:uid="{00000000-0004-0000-0000-000012000000}"/>
+    <hyperlink ref="S21" r:id="rId20" xr:uid="{00000000-0004-0000-0000-000013000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+  <pageSetup orientation="portrait" useFirstPageNumber="1" horizontalDpi="4294967295" verticalDpi="4294967295"/>
   <headerFooter>
     <oddFooter>&amp;L_x000D_&amp;1#&amp;"Calibri"&amp;10&amp;K000000 EXPLEO Internal</oddFooter>
   </headerFooter>

</xml_diff>